<commit_message>
chore: remove a file
</commit_message>
<xml_diff>
--- a/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/Planning prévisionnel Habilitations Nucléaires 3 Ok.xlsx
+++ b/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/Planning prévisionnel Habilitations Nucléaires 3 Ok.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\18_Bourges\Collaborateurs\Christophe HAMEL\Lot 2 Habilitation Nucléaire Ouzouer sur Loire\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E929FCC-ACDD-47E0-A12F-F4FC7BA36476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D17A5247-4B7E-4F2D-8051-B78F30B21410}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D17A5247-4B7E-4F2D-8051-B78F30B21410}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -1038,6 +1038,72 @@
     <xf numFmtId="0" fontId="2" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1054,72 +1120,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1460,51 +1460,51 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:AQ49"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="2.33203125" customWidth="1"/>
-    <col min="3" max="3" width="6.5546875" customWidth="1"/>
-    <col min="4" max="4" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.88671875" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" customWidth="1"/>
-    <col min="8" max="8" width="2.5546875" customWidth="1"/>
-    <col min="9" max="9" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.6640625" customWidth="1"/>
-    <col min="13" max="13" width="6.44140625" customWidth="1"/>
-    <col min="14" max="14" width="2.33203125" customWidth="1"/>
-    <col min="15" max="15" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.44140625" customWidth="1"/>
-    <col min="17" max="17" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.5546875" customWidth="1"/>
-    <col min="19" max="19" width="5.109375" customWidth="1"/>
-    <col min="20" max="20" width="2.5546875" customWidth="1"/>
-    <col min="21" max="21" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.44140625" customWidth="1"/>
-    <col min="23" max="23" width="20.5546875" customWidth="1"/>
-    <col min="24" max="24" width="5.44140625" customWidth="1"/>
-    <col min="25" max="25" width="4.88671875" customWidth="1"/>
-    <col min="26" max="26" width="2.33203125" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="20.5546875" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="11.44140625" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="5.6640625" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="5.44140625" hidden="1" customWidth="1"/>
-    <col min="32" max="32" width="2.6640625" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="6.6640625" hidden="1" customWidth="1"/>
-    <col min="34" max="35" width="11.44140625" hidden="1" customWidth="1"/>
-    <col min="36" max="36" width="6.109375" hidden="1" customWidth="1"/>
-    <col min="37" max="37" width="5.5546875" hidden="1" customWidth="1"/>
-    <col min="38" max="38" width="2.5546875" hidden="1" customWidth="1"/>
-    <col min="39" max="39" width="6.5546875" hidden="1" customWidth="1"/>
-    <col min="40" max="41" width="11.44140625" hidden="1" customWidth="1"/>
-    <col min="42" max="42" width="6.5546875" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="2.28515625" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" customWidth="1"/>
+    <col min="4" max="4" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.85546875" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" customWidth="1"/>
+    <col min="8" max="8" width="2.5703125" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.7109375" customWidth="1"/>
+    <col min="13" max="13" width="6.42578125" customWidth="1"/>
+    <col min="14" max="14" width="2.28515625" customWidth="1"/>
+    <col min="15" max="15" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.42578125" customWidth="1"/>
+    <col min="17" max="17" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.5703125" customWidth="1"/>
+    <col min="19" max="19" width="5.140625" customWidth="1"/>
+    <col min="20" max="20" width="2.5703125" customWidth="1"/>
+    <col min="21" max="21" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" customWidth="1"/>
+    <col min="23" max="23" width="20.5703125" customWidth="1"/>
+    <col min="24" max="24" width="5.42578125" customWidth="1"/>
+    <col min="25" max="25" width="4.85546875" customWidth="1"/>
+    <col min="26" max="26" width="2.28515625" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="7.28515625" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="20.5703125" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="11.42578125" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="5.7109375" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="5.42578125" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="2.7109375" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="6.7109375" hidden="1" customWidth="1"/>
+    <col min="34" max="35" width="11.42578125" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="6.140625" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="5.5703125" hidden="1" customWidth="1"/>
+    <col min="38" max="38" width="2.5703125" hidden="1" customWidth="1"/>
+    <col min="39" max="39" width="6.5703125" hidden="1" customWidth="1"/>
+    <col min="40" max="41" width="11.42578125" hidden="1" customWidth="1"/>
+    <col min="42" max="42" width="6.5703125" hidden="1" customWidth="1"/>
     <col min="43" max="43" width="6" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:43" s="22" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:43" s="22" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="C2" s="23" t="s">
         <v>43</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="3" spans="2:43" s="22" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:43" s="22" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="C3" s="23" t="s">
         <v>44</v>
       </c>
@@ -1526,7 +1526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:43" s="22" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:43" s="22" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="C4" s="23" t="s">
         <v>45</v>
       </c>
@@ -1538,8 +1538,8 @@
         <v>245</v>
       </c>
     </row>
-    <row r="5" spans="2:43" s="22" customFormat="1" ht="21" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:43" s="22" customFormat="1" ht="21" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B6" s="62"/>
       <c r="C6" s="63"/>
       <c r="D6" s="63" t="s">
@@ -1548,54 +1548,54 @@
       <c r="E6" s="63"/>
       <c r="F6" s="63"/>
       <c r="G6" s="61"/>
-      <c r="H6" s="109" t="s">
+      <c r="H6" s="100" t="s">
         <v>3</v>
       </c>
-      <c r="I6" s="109"/>
-      <c r="J6" s="109"/>
-      <c r="K6" s="109"/>
-      <c r="L6" s="109"/>
-      <c r="M6" s="109"/>
-      <c r="N6" s="109" t="s">
+      <c r="I6" s="100"/>
+      <c r="J6" s="100"/>
+      <c r="K6" s="100"/>
+      <c r="L6" s="100"/>
+      <c r="M6" s="100"/>
+      <c r="N6" s="100" t="s">
         <v>4</v>
       </c>
-      <c r="O6" s="109"/>
-      <c r="P6" s="109"/>
-      <c r="Q6" s="109"/>
-      <c r="R6" s="109"/>
-      <c r="S6" s="109"/>
-      <c r="T6" s="113"/>
-      <c r="U6" s="113"/>
-      <c r="V6" s="113"/>
-      <c r="W6" s="113"/>
-      <c r="X6" s="113"/>
-      <c r="Y6" s="113"/>
-      <c r="Z6" s="115" t="s">
+      <c r="O6" s="100"/>
+      <c r="P6" s="100"/>
+      <c r="Q6" s="100"/>
+      <c r="R6" s="100"/>
+      <c r="S6" s="100"/>
+      <c r="T6" s="115"/>
+      <c r="U6" s="115"/>
+      <c r="V6" s="115"/>
+      <c r="W6" s="115"/>
+      <c r="X6" s="115"/>
+      <c r="Y6" s="115"/>
+      <c r="Z6" s="116" t="s">
         <v>4</v>
       </c>
-      <c r="AA6" s="109"/>
-      <c r="AB6" s="109"/>
-      <c r="AC6" s="109"/>
-      <c r="AD6" s="109"/>
-      <c r="AE6" s="109"/>
-      <c r="AF6" s="109" t="s">
+      <c r="AA6" s="100"/>
+      <c r="AB6" s="100"/>
+      <c r="AC6" s="100"/>
+      <c r="AD6" s="100"/>
+      <c r="AE6" s="100"/>
+      <c r="AF6" s="100" t="s">
         <v>5</v>
       </c>
-      <c r="AG6" s="109"/>
-      <c r="AH6" s="109"/>
-      <c r="AI6" s="109"/>
-      <c r="AJ6" s="109"/>
-      <c r="AK6" s="109"/>
-      <c r="AL6" s="109" t="s">
+      <c r="AG6" s="100"/>
+      <c r="AH6" s="100"/>
+      <c r="AI6" s="100"/>
+      <c r="AJ6" s="100"/>
+      <c r="AK6" s="100"/>
+      <c r="AL6" s="100" t="s">
         <v>6</v>
       </c>
-      <c r="AM6" s="109"/>
-      <c r="AN6" s="109"/>
-      <c r="AO6" s="109"/>
-      <c r="AP6" s="109"/>
-      <c r="AQ6" s="109"/>
-    </row>
-    <row r="7" spans="2:43" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AM6" s="100"/>
+      <c r="AN6" s="100"/>
+      <c r="AO6" s="100"/>
+      <c r="AP6" s="100"/>
+      <c r="AQ6" s="100"/>
+    </row>
+    <row r="7" spans="2:43" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="13"/>
       <c r="C7" s="6"/>
       <c r="D7" s="7" t="s">
@@ -1687,7 +1687,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="46"/>
       <c r="C8" s="12">
         <v>45992</v>
@@ -1696,16 +1696,16 @@
       <c r="E8" s="28"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="110" t="s">
+      <c r="H8" s="101" t="s">
         <v>14</v>
       </c>
       <c r="I8" s="21">
         <v>46023</v>
       </c>
-      <c r="J8" s="116" t="s">
+      <c r="J8" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="117"/>
+      <c r="K8" s="104"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
       <c r="N8" s="8"/>
@@ -1716,10 +1716,10 @@
       <c r="Q8" s="14"/>
       <c r="R8" s="15"/>
       <c r="S8" s="15"/>
-      <c r="T8" s="114"/>
+      <c r="T8" s="96"/>
       <c r="U8" s="71"/>
-      <c r="V8" s="112"/>
-      <c r="W8" s="112"/>
+      <c r="V8" s="114"/>
+      <c r="W8" s="114"/>
       <c r="X8" s="73"/>
       <c r="Y8" s="73"/>
       <c r="Z8" s="66"/>
@@ -1738,7 +1738,7 @@
       <c r="AI8" s="14"/>
       <c r="AJ8" s="15"/>
       <c r="AK8" s="15"/>
-      <c r="AL8" s="110" t="s">
+      <c r="AL8" s="101" t="s">
         <v>15</v>
       </c>
       <c r="AM8" s="12">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="AQ8" s="2"/>
     </row>
-    <row r="9" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B9" s="60"/>
       <c r="C9" s="12">
         <v>45993</v>
@@ -1762,7 +1762,7 @@
       <c r="E9" s="29"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="110"/>
+      <c r="H9" s="101"/>
       <c r="I9" s="21">
         <v>46024</v>
       </c>
@@ -1770,7 +1770,7 @@
       <c r="K9" s="14"/>
       <c r="L9" s="33"/>
       <c r="M9" s="34"/>
-      <c r="N9" s="110" t="s">
+      <c r="N9" s="101" t="s">
         <v>16</v>
       </c>
       <c r="O9" s="1">
@@ -1786,13 +1786,13 @@
         <v>7</v>
       </c>
       <c r="S9" s="2"/>
-      <c r="T9" s="114"/>
+      <c r="T9" s="96"/>
       <c r="U9" s="71"/>
       <c r="V9" s="71"/>
       <c r="W9" s="71"/>
       <c r="X9" s="74"/>
       <c r="Y9" s="74"/>
-      <c r="Z9" s="111" t="s">
+      <c r="Z9" s="99" t="s">
         <v>16</v>
       </c>
       <c r="AA9" s="1">
@@ -1806,7 +1806,7 @@
         <v>7</v>
       </c>
       <c r="AE9" s="2"/>
-      <c r="AF9" s="110" t="s">
+      <c r="AF9" s="101" t="s">
         <v>17</v>
       </c>
       <c r="AG9" s="12">
@@ -1820,7 +1820,7 @@
       <c r="AK9" s="2">
         <v>7</v>
       </c>
-      <c r="AL9" s="110"/>
+      <c r="AL9" s="101"/>
       <c r="AM9" s="12">
         <v>46114</v>
       </c>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="AQ9" s="2"/>
     </row>
-    <row r="10" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="60"/>
       <c r="C10" s="12">
         <v>45994</v>
@@ -1842,7 +1842,7 @@
       <c r="E10" s="29"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
-      <c r="H10" s="110"/>
+      <c r="H10" s="101"/>
       <c r="I10" s="21">
         <v>46025</v>
       </c>
@@ -1850,7 +1850,7 @@
       <c r="K10" s="14"/>
       <c r="L10" s="15"/>
       <c r="M10" s="20"/>
-      <c r="N10" s="110"/>
+      <c r="N10" s="101"/>
       <c r="O10" s="1">
         <v>46056</v>
       </c>
@@ -1864,13 +1864,13 @@
         <v>7</v>
       </c>
       <c r="S10" s="2"/>
-      <c r="T10" s="114"/>
+      <c r="T10" s="96"/>
       <c r="U10" s="71"/>
       <c r="V10" s="71"/>
       <c r="W10" s="71"/>
       <c r="X10" s="75"/>
       <c r="Y10" s="75"/>
-      <c r="Z10" s="111"/>
+      <c r="Z10" s="99"/>
       <c r="AA10" s="1">
         <v>46056</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>7</v>
       </c>
       <c r="AE10" s="2"/>
-      <c r="AF10" s="110"/>
+      <c r="AF10" s="101"/>
       <c r="AG10" s="12">
         <v>46084</v>
       </c>
@@ -1894,7 +1894,7 @@
       <c r="AK10" s="2">
         <v>7</v>
       </c>
-      <c r="AL10" s="110"/>
+      <c r="AL10" s="101"/>
       <c r="AM10" s="12">
         <v>46115</v>
       </c>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="AQ10" s="2"/>
     </row>
-    <row r="11" spans="2:43" ht="18" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:43" ht="19.5" x14ac:dyDescent="0.25">
       <c r="B11" s="60" t="s">
         <v>12</v>
       </c>
@@ -1918,7 +1918,7 @@
       <c r="E11" s="29"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="110"/>
+      <c r="H11" s="101"/>
       <c r="I11" s="21">
         <v>46026</v>
       </c>
@@ -1926,7 +1926,7 @@
       <c r="K11" s="14"/>
       <c r="L11" s="15"/>
       <c r="M11" s="20"/>
-      <c r="N11" s="110"/>
+      <c r="N11" s="101"/>
       <c r="O11" s="1">
         <v>46057</v>
       </c>
@@ -1940,13 +1940,13 @@
         <v>7</v>
       </c>
       <c r="S11" s="2"/>
-      <c r="T11" s="114"/>
+      <c r="T11" s="96"/>
       <c r="U11" s="71"/>
       <c r="V11" s="71"/>
       <c r="W11" s="71"/>
       <c r="X11" s="75"/>
       <c r="Y11" s="75"/>
-      <c r="Z11" s="111"/>
+      <c r="Z11" s="99"/>
       <c r="AA11" s="1">
         <v>46057</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>7</v>
       </c>
       <c r="AE11" s="2"/>
-      <c r="AF11" s="110"/>
+      <c r="AF11" s="101"/>
       <c r="AG11" s="12">
         <v>46085</v>
       </c>
@@ -1970,7 +1970,7 @@
       <c r="AK11" s="2">
         <v>7</v>
       </c>
-      <c r="AL11" s="110"/>
+      <c r="AL11" s="101"/>
       <c r="AM11" s="21">
         <v>46116</v>
       </c>
@@ -1979,7 +1979,7 @@
       <c r="AP11" s="15"/>
       <c r="AQ11" s="15"/>
     </row>
-    <row r="12" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B12" s="60"/>
       <c r="C12" s="12">
         <v>45996</v>
@@ -1988,7 +1988,7 @@
       <c r="E12" s="29"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="110" t="s">
+      <c r="H12" s="101" t="s">
         <v>18</v>
       </c>
       <c r="I12" s="12">
@@ -2004,7 +2004,7 @@
         <v>7</v>
       </c>
       <c r="M12" s="2"/>
-      <c r="N12" s="110"/>
+      <c r="N12" s="101"/>
       <c r="O12" s="1">
         <v>46058</v>
       </c>
@@ -2018,13 +2018,13 @@
         <v>7</v>
       </c>
       <c r="S12" s="2"/>
-      <c r="T12" s="114"/>
+      <c r="T12" s="96"/>
       <c r="U12" s="71"/>
       <c r="V12" s="76"/>
       <c r="W12" s="71"/>
       <c r="X12" s="75"/>
       <c r="Y12" s="75"/>
-      <c r="Z12" s="111"/>
+      <c r="Z12" s="99"/>
       <c r="AA12" s="1">
         <v>46058</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>7</v>
       </c>
       <c r="AE12" s="2"/>
-      <c r="AF12" s="110"/>
+      <c r="AF12" s="101"/>
       <c r="AG12" s="12">
         <v>46086</v>
       </c>
@@ -2048,7 +2048,7 @@
       <c r="AK12" s="2">
         <v>7</v>
       </c>
-      <c r="AL12" s="110"/>
+      <c r="AL12" s="101"/>
       <c r="AM12" s="21">
         <v>46117</v>
       </c>
@@ -2057,7 +2057,7 @@
       <c r="AP12" s="15"/>
       <c r="AQ12" s="15"/>
     </row>
-    <row r="13" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="60"/>
       <c r="C13" s="21">
         <v>45997</v>
@@ -2066,7 +2066,7 @@
       <c r="E13" s="30"/>
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
-      <c r="H13" s="110"/>
+      <c r="H13" s="101"/>
       <c r="I13" s="12">
         <v>46028</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>7</v>
       </c>
       <c r="M13" s="2"/>
-      <c r="N13" s="110"/>
+      <c r="N13" s="101"/>
       <c r="O13" s="1">
         <v>46059</v>
       </c>
@@ -2092,13 +2092,13 @@
         <v>7</v>
       </c>
       <c r="S13" s="2"/>
-      <c r="T13" s="114"/>
+      <c r="T13" s="96"/>
       <c r="U13" s="71"/>
       <c r="V13" s="76"/>
       <c r="W13" s="71"/>
       <c r="X13" s="75"/>
       <c r="Y13" s="75"/>
-      <c r="Z13" s="111"/>
+      <c r="Z13" s="99"/>
       <c r="AA13" s="1">
         <v>46059</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>7</v>
       </c>
       <c r="AE13" s="2"/>
-      <c r="AF13" s="110"/>
+      <c r="AF13" s="101"/>
       <c r="AG13" s="12">
         <v>46087</v>
       </c>
@@ -2122,20 +2122,20 @@
       <c r="AK13" s="2">
         <v>7</v>
       </c>
-      <c r="AL13" s="110" t="s">
+      <c r="AL13" s="101" t="s">
         <v>21</v>
       </c>
       <c r="AM13" s="21">
         <v>46118</v>
       </c>
-      <c r="AN13" s="116" t="s">
+      <c r="AN13" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="AO13" s="121"/>
+      <c r="AO13" s="103"/>
       <c r="AP13" s="15"/>
       <c r="AQ13" s="15"/>
     </row>
-    <row r="14" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B14" s="47"/>
       <c r="C14" s="21">
         <v>45998</v>
@@ -2144,7 +2144,7 @@
       <c r="E14" s="21"/>
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
-      <c r="H14" s="110"/>
+      <c r="H14" s="101"/>
       <c r="I14" s="12">
         <v>46029</v>
       </c>
@@ -2156,7 +2156,7 @@
         <v>7</v>
       </c>
       <c r="M14" s="2"/>
-      <c r="N14" s="110"/>
+      <c r="N14" s="101"/>
       <c r="O14" s="14">
         <v>46060</v>
       </c>
@@ -2164,13 +2164,13 @@
       <c r="Q14" s="14"/>
       <c r="R14" s="15"/>
       <c r="S14" s="15"/>
-      <c r="T14" s="114"/>
+      <c r="T14" s="96"/>
       <c r="U14" s="71"/>
       <c r="V14" s="76"/>
       <c r="W14" s="71"/>
       <c r="X14" s="75"/>
       <c r="Y14" s="75"/>
-      <c r="Z14" s="111"/>
+      <c r="Z14" s="99"/>
       <c r="AA14" s="14">
         <v>46060</v>
       </c>
@@ -2178,7 +2178,7 @@
       <c r="AC14" s="14"/>
       <c r="AD14" s="15"/>
       <c r="AE14" s="15"/>
-      <c r="AF14" s="110"/>
+      <c r="AF14" s="101"/>
       <c r="AG14" s="21">
         <v>46088</v>
       </c>
@@ -2186,7 +2186,7 @@
       <c r="AI14" s="14"/>
       <c r="AJ14" s="15"/>
       <c r="AK14" s="15"/>
-      <c r="AL14" s="110"/>
+      <c r="AL14" s="101"/>
       <c r="AM14" s="12">
         <v>46119</v>
       </c>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="AQ14" s="2"/>
     </row>
-    <row r="15" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="46"/>
       <c r="C15" s="12">
         <v>45999</v>
@@ -2208,7 +2208,7 @@
       <c r="E15" s="31"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="110"/>
+      <c r="H15" s="101"/>
       <c r="I15" s="12">
         <v>46030</v>
       </c>
@@ -2220,7 +2220,7 @@
         <v>7</v>
       </c>
       <c r="M15" s="2"/>
-      <c r="N15" s="110"/>
+      <c r="N15" s="101"/>
       <c r="O15" s="14">
         <v>46061</v>
       </c>
@@ -2228,13 +2228,13 @@
       <c r="Q15" s="18"/>
       <c r="R15" s="18"/>
       <c r="S15" s="18"/>
-      <c r="T15" s="114"/>
+      <c r="T15" s="96"/>
       <c r="U15" s="71"/>
       <c r="V15" s="76"/>
       <c r="W15" s="71"/>
       <c r="X15" s="75"/>
       <c r="Y15" s="75"/>
-      <c r="Z15" s="111"/>
+      <c r="Z15" s="99"/>
       <c r="AA15" s="14">
         <v>46061</v>
       </c>
@@ -2242,7 +2242,7 @@
       <c r="AC15" s="18"/>
       <c r="AD15" s="18"/>
       <c r="AE15" s="18"/>
-      <c r="AF15" s="110"/>
+      <c r="AF15" s="101"/>
       <c r="AG15" s="21">
         <v>46089</v>
       </c>
@@ -2250,7 +2250,7 @@
       <c r="AI15" s="18"/>
       <c r="AJ15" s="18"/>
       <c r="AK15" s="18"/>
-      <c r="AL15" s="110"/>
+      <c r="AL15" s="101"/>
       <c r="AM15" s="12">
         <v>46120</v>
       </c>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="AQ15" s="4"/>
     </row>
-    <row r="16" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B16" s="60"/>
       <c r="C16" s="12">
         <v>46000</v>
@@ -2272,7 +2272,7 @@
       <c r="E16" s="29"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="110"/>
+      <c r="H16" s="101"/>
       <c r="I16" s="12">
         <v>46031</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>7</v>
       </c>
       <c r="M16" s="2"/>
-      <c r="N16" s="110" t="s">
+      <c r="N16" s="101" t="s">
         <v>26</v>
       </c>
       <c r="O16" s="1">
@@ -2300,13 +2300,13 @@
         <v>7</v>
       </c>
       <c r="S16" s="2"/>
-      <c r="T16" s="114"/>
+      <c r="T16" s="96"/>
       <c r="U16" s="71"/>
       <c r="V16" s="76"/>
       <c r="W16" s="71"/>
       <c r="X16" s="75"/>
       <c r="Y16" s="75"/>
-      <c r="Z16" s="111" t="s">
+      <c r="Z16" s="99" t="s">
         <v>26</v>
       </c>
       <c r="AA16" s="1">
@@ -2320,7 +2320,7 @@
         <v>7</v>
       </c>
       <c r="AE16" s="2"/>
-      <c r="AF16" s="110" t="s">
+      <c r="AF16" s="101" t="s">
         <v>27</v>
       </c>
       <c r="AG16" s="12">
@@ -2334,7 +2334,7 @@
         <v>7</v>
       </c>
       <c r="AK16" s="2"/>
-      <c r="AL16" s="110"/>
+      <c r="AL16" s="101"/>
       <c r="AM16" s="12">
         <v>46121</v>
       </c>
@@ -2343,7 +2343,7 @@
       <c r="AP16" s="2"/>
       <c r="AQ16" s="2"/>
     </row>
-    <row r="17" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="60"/>
       <c r="C17" s="12">
         <v>46001</v>
@@ -2352,7 +2352,7 @@
       <c r="E17" s="29"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
-      <c r="H17" s="110"/>
+      <c r="H17" s="101"/>
       <c r="I17" s="21">
         <v>46032</v>
       </c>
@@ -2360,7 +2360,7 @@
       <c r="K17" s="14"/>
       <c r="L17" s="15"/>
       <c r="M17" s="20"/>
-      <c r="N17" s="110"/>
+      <c r="N17" s="101"/>
       <c r="O17" s="1">
         <v>46063</v>
       </c>
@@ -2374,13 +2374,13 @@
         <v>7</v>
       </c>
       <c r="S17" s="2"/>
-      <c r="T17" s="114"/>
+      <c r="T17" s="96"/>
       <c r="U17" s="71"/>
       <c r="V17" s="71"/>
       <c r="W17" s="71"/>
       <c r="X17" s="75"/>
       <c r="Y17" s="75"/>
-      <c r="Z17" s="111"/>
+      <c r="Z17" s="99"/>
       <c r="AA17" s="1">
         <v>46063</v>
       </c>
@@ -2392,7 +2392,7 @@
         <v>7</v>
       </c>
       <c r="AE17" s="2"/>
-      <c r="AF17" s="110"/>
+      <c r="AF17" s="101"/>
       <c r="AG17" s="12">
         <v>46091</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>7</v>
       </c>
       <c r="AK17" s="2"/>
-      <c r="AL17" s="110"/>
+      <c r="AL17" s="101"/>
       <c r="AM17" s="12">
         <v>46122</v>
       </c>
@@ -2413,7 +2413,7 @@
       <c r="AP17" s="2"/>
       <c r="AQ17" s="2"/>
     </row>
-    <row r="18" spans="2:43" ht="18" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:43" ht="19.5" x14ac:dyDescent="0.25">
       <c r="B18" s="60" t="s">
         <v>24</v>
       </c>
@@ -2424,7 +2424,7 @@
       <c r="E18" s="28"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="110"/>
+      <c r="H18" s="101"/>
       <c r="I18" s="21">
         <v>46033</v>
       </c>
@@ -2432,7 +2432,7 @@
       <c r="K18" s="16"/>
       <c r="L18" s="16"/>
       <c r="M18" s="36"/>
-      <c r="N18" s="110"/>
+      <c r="N18" s="101"/>
       <c r="O18" s="1">
         <v>46064</v>
       </c>
@@ -2446,13 +2446,13 @@
         <v>7</v>
       </c>
       <c r="S18" s="2"/>
-      <c r="T18" s="114"/>
+      <c r="T18" s="96"/>
       <c r="U18" s="71"/>
       <c r="V18" s="73"/>
       <c r="W18" s="73"/>
       <c r="X18" s="73"/>
       <c r="Y18" s="73"/>
-      <c r="Z18" s="111"/>
+      <c r="Z18" s="99"/>
       <c r="AA18" s="1">
         <v>46064</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>7</v>
       </c>
       <c r="AE18" s="2"/>
-      <c r="AF18" s="110"/>
+      <c r="AF18" s="101"/>
       <c r="AG18" s="12">
         <v>46092</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>7</v>
       </c>
       <c r="AK18" s="2"/>
-      <c r="AL18" s="110"/>
+      <c r="AL18" s="101"/>
       <c r="AM18" s="21">
         <v>46123</v>
       </c>
@@ -2485,7 +2485,7 @@
       <c r="AP18" s="15"/>
       <c r="AQ18" s="15"/>
     </row>
-    <row r="19" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B19" s="60"/>
       <c r="C19" s="12">
         <v>46003</v>
@@ -2494,7 +2494,7 @@
       <c r="E19" s="29"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
-      <c r="H19" s="110" t="s">
+      <c r="H19" s="101" t="s">
         <v>29</v>
       </c>
       <c r="I19" s="12">
@@ -2508,7 +2508,7 @@
         <v>7</v>
       </c>
       <c r="M19" s="35"/>
-      <c r="N19" s="110"/>
+      <c r="N19" s="101"/>
       <c r="O19" s="1">
         <v>46065</v>
       </c>
@@ -2522,13 +2522,13 @@
         <v>7</v>
       </c>
       <c r="S19" s="2"/>
-      <c r="T19" s="114"/>
+      <c r="T19" s="96"/>
       <c r="U19" s="71"/>
       <c r="V19" s="76"/>
       <c r="W19" s="71"/>
       <c r="X19" s="75"/>
       <c r="Y19" s="75"/>
-      <c r="Z19" s="111"/>
+      <c r="Z19" s="99"/>
       <c r="AA19" s="1">
         <v>46065</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>7</v>
       </c>
       <c r="AE19" s="2"/>
-      <c r="AF19" s="110"/>
+      <c r="AF19" s="101"/>
       <c r="AG19" s="12">
         <v>46093</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>7</v>
       </c>
       <c r="AK19" s="2"/>
-      <c r="AL19" s="110"/>
+      <c r="AL19" s="101"/>
       <c r="AM19" s="21">
         <v>46124</v>
       </c>
@@ -2561,7 +2561,7 @@
       <c r="AP19" s="15"/>
       <c r="AQ19" s="15"/>
     </row>
-    <row r="20" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="60"/>
       <c r="C20" s="21">
         <v>46004</v>
@@ -2570,7 +2570,7 @@
       <c r="E20" s="17"/>
       <c r="F20" s="15"/>
       <c r="G20" s="15"/>
-      <c r="H20" s="110"/>
+      <c r="H20" s="101"/>
       <c r="I20" s="12">
         <v>46035</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>7</v>
       </c>
       <c r="M20" s="35"/>
-      <c r="N20" s="110"/>
+      <c r="N20" s="101"/>
       <c r="O20" s="1">
         <v>46066</v>
       </c>
@@ -2594,13 +2594,13 @@
         <v>7</v>
       </c>
       <c r="S20" s="2"/>
-      <c r="T20" s="114"/>
+      <c r="T20" s="96"/>
       <c r="U20" s="71"/>
       <c r="V20" s="76"/>
       <c r="W20" s="76"/>
       <c r="X20" s="75"/>
       <c r="Y20" s="75"/>
-      <c r="Z20" s="111"/>
+      <c r="Z20" s="99"/>
       <c r="AA20" s="1">
         <v>46066</v>
       </c>
@@ -2612,7 +2612,7 @@
         <v>7</v>
       </c>
       <c r="AE20" s="2"/>
-      <c r="AF20" s="110"/>
+      <c r="AF20" s="101"/>
       <c r="AG20" s="12">
         <v>46094</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>7</v>
       </c>
       <c r="AK20" s="2"/>
-      <c r="AL20" s="110" t="s">
+      <c r="AL20" s="101" t="s">
         <v>30</v>
       </c>
       <c r="AM20" s="12">
@@ -2635,7 +2635,7 @@
       <c r="AP20" s="2"/>
       <c r="AQ20" s="2"/>
     </row>
-    <row r="21" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B21" s="47"/>
       <c r="C21" s="21">
         <v>46005</v>
@@ -2644,7 +2644,7 @@
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
-      <c r="H21" s="110"/>
+      <c r="H21" s="101"/>
       <c r="I21" s="12">
         <v>46036</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>7</v>
       </c>
       <c r="M21" s="35"/>
-      <c r="N21" s="110"/>
+      <c r="N21" s="101"/>
       <c r="O21" s="14">
         <v>46067</v>
       </c>
@@ -2664,13 +2664,13 @@
       <c r="Q21" s="14"/>
       <c r="R21" s="15"/>
       <c r="S21" s="15"/>
-      <c r="T21" s="114"/>
+      <c r="T21" s="96"/>
       <c r="U21" s="71"/>
       <c r="V21" s="76"/>
       <c r="W21" s="76"/>
       <c r="X21" s="75"/>
       <c r="Y21" s="75"/>
-      <c r="Z21" s="111"/>
+      <c r="Z21" s="99"/>
       <c r="AA21" s="14">
         <v>46067</v>
       </c>
@@ -2678,7 +2678,7 @@
       <c r="AC21" s="14"/>
       <c r="AD21" s="15"/>
       <c r="AE21" s="15"/>
-      <c r="AF21" s="110"/>
+      <c r="AF21" s="101"/>
       <c r="AG21" s="21">
         <v>46095</v>
       </c>
@@ -2686,7 +2686,7 @@
       <c r="AI21" s="14"/>
       <c r="AJ21" s="15"/>
       <c r="AK21" s="15"/>
-      <c r="AL21" s="110"/>
+      <c r="AL21" s="101"/>
       <c r="AM21" s="12">
         <v>46126</v>
       </c>
@@ -2695,7 +2695,7 @@
       <c r="AP21" s="2"/>
       <c r="AQ21" s="2"/>
     </row>
-    <row r="22" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="46"/>
       <c r="C22" s="12">
         <v>46006</v>
@@ -2710,7 +2710,7 @@
         <v>7</v>
       </c>
       <c r="G22" s="2"/>
-      <c r="H22" s="110"/>
+      <c r="H22" s="101"/>
       <c r="I22" s="12">
         <v>46037</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>7</v>
       </c>
       <c r="M22" s="35"/>
-      <c r="N22" s="110"/>
+      <c r="N22" s="101"/>
       <c r="O22" s="14">
         <v>46068</v>
       </c>
@@ -2730,13 +2730,13 @@
       <c r="Q22" s="14"/>
       <c r="R22" s="15"/>
       <c r="S22" s="15"/>
-      <c r="T22" s="114"/>
+      <c r="T22" s="96"/>
       <c r="U22" s="71"/>
       <c r="V22" s="76"/>
       <c r="W22" s="76"/>
       <c r="X22" s="75"/>
       <c r="Y22" s="75"/>
-      <c r="Z22" s="111"/>
+      <c r="Z22" s="99"/>
       <c r="AA22" s="14">
         <v>46068</v>
       </c>
@@ -2744,7 +2744,7 @@
       <c r="AC22" s="14"/>
       <c r="AD22" s="15"/>
       <c r="AE22" s="15"/>
-      <c r="AF22" s="110"/>
+      <c r="AF22" s="101"/>
       <c r="AG22" s="21">
         <v>46096</v>
       </c>
@@ -2752,7 +2752,7 @@
       <c r="AI22" s="14"/>
       <c r="AJ22" s="15"/>
       <c r="AK22" s="15"/>
-      <c r="AL22" s="110"/>
+      <c r="AL22" s="101"/>
       <c r="AM22" s="12">
         <v>46127</v>
       </c>
@@ -2761,7 +2761,7 @@
       <c r="AP22" s="2"/>
       <c r="AQ22" s="2"/>
     </row>
-    <row r="23" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B23" s="60"/>
       <c r="C23" s="12">
         <v>46007</v>
@@ -2776,7 +2776,7 @@
         <v>7</v>
       </c>
       <c r="G23" s="2"/>
-      <c r="H23" s="110"/>
+      <c r="H23" s="101"/>
       <c r="I23" s="12">
         <v>46038</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>7</v>
       </c>
       <c r="M23" s="35"/>
-      <c r="N23" s="110" t="s">
+      <c r="N23" s="101" t="s">
         <v>32</v>
       </c>
       <c r="O23" s="1">
@@ -2800,13 +2800,13 @@
       <c r="Q23" s="3"/>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
-      <c r="T23" s="114"/>
+      <c r="T23" s="96"/>
       <c r="U23" s="71"/>
       <c r="V23" s="76"/>
       <c r="W23" s="71"/>
       <c r="X23" s="75"/>
       <c r="Y23" s="75"/>
-      <c r="Z23" s="111" t="s">
+      <c r="Z23" s="99" t="s">
         <v>32</v>
       </c>
       <c r="AA23" s="1">
@@ -2820,7 +2820,7 @@
       <c r="AE23" s="2">
         <v>7</v>
       </c>
-      <c r="AF23" s="110" t="s">
+      <c r="AF23" s="101" t="s">
         <v>33</v>
       </c>
       <c r="AG23" s="12">
@@ -2834,7 +2834,7 @@
         <v>7</v>
       </c>
       <c r="AK23" s="2"/>
-      <c r="AL23" s="110"/>
+      <c r="AL23" s="101"/>
       <c r="AM23" s="12">
         <v>46128</v>
       </c>
@@ -2843,7 +2843,7 @@
       <c r="AP23" s="2"/>
       <c r="AQ23" s="2"/>
     </row>
-    <row r="24" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="60"/>
       <c r="C24" s="12">
         <v>46008</v>
@@ -2858,7 +2858,7 @@
         <v>7</v>
       </c>
       <c r="G24" s="2"/>
-      <c r="H24" s="110"/>
+      <c r="H24" s="101"/>
       <c r="I24" s="21">
         <v>46039</v>
       </c>
@@ -2866,7 +2866,7 @@
       <c r="K24" s="14"/>
       <c r="L24" s="15"/>
       <c r="M24" s="20"/>
-      <c r="N24" s="110"/>
+      <c r="N24" s="101"/>
       <c r="O24" s="1">
         <v>46070</v>
       </c>
@@ -2874,13 +2874,13 @@
       <c r="Q24" s="3"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
-      <c r="T24" s="114"/>
+      <c r="T24" s="96"/>
       <c r="U24" s="71"/>
       <c r="V24" s="71"/>
       <c r="W24" s="71"/>
       <c r="X24" s="75"/>
       <c r="Y24" s="75"/>
-      <c r="Z24" s="111"/>
+      <c r="Z24" s="99"/>
       <c r="AA24" s="1">
         <v>46070</v>
       </c>
@@ -2892,7 +2892,7 @@
       <c r="AE24" s="2">
         <v>7</v>
       </c>
-      <c r="AF24" s="110"/>
+      <c r="AF24" s="101"/>
       <c r="AG24" s="12">
         <v>46098</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>7</v>
       </c>
       <c r="AK24" s="2"/>
-      <c r="AL24" s="110"/>
+      <c r="AL24" s="101"/>
       <c r="AM24" s="12">
         <v>46129</v>
       </c>
@@ -2913,7 +2913,7 @@
       <c r="AP24" s="2"/>
       <c r="AQ24" s="2"/>
     </row>
-    <row r="25" spans="2:43" ht="18" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:43" ht="19.5" x14ac:dyDescent="0.25">
       <c r="B25" s="60" t="s">
         <v>31</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>7</v>
       </c>
       <c r="G25" s="2"/>
-      <c r="H25" s="110"/>
+      <c r="H25" s="101"/>
       <c r="I25" s="21">
         <v>46040</v>
       </c>
@@ -2938,7 +2938,7 @@
       <c r="K25" s="17"/>
       <c r="L25" s="15"/>
       <c r="M25" s="26"/>
-      <c r="N25" s="110"/>
+      <c r="N25" s="101"/>
       <c r="O25" s="1">
         <v>46071</v>
       </c>
@@ -2946,13 +2946,13 @@
       <c r="Q25" s="3"/>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
-      <c r="T25" s="114"/>
+      <c r="T25" s="96"/>
       <c r="U25" s="71"/>
       <c r="V25" s="76"/>
       <c r="W25" s="76"/>
       <c r="X25" s="75"/>
       <c r="Y25" s="72"/>
-      <c r="Z25" s="111"/>
+      <c r="Z25" s="99"/>
       <c r="AA25" s="1">
         <v>46071</v>
       </c>
@@ -2964,7 +2964,7 @@
       <c r="AE25" s="2">
         <v>7</v>
       </c>
-      <c r="AF25" s="110"/>
+      <c r="AF25" s="101"/>
       <c r="AG25" s="12">
         <v>46099</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>7</v>
       </c>
       <c r="AK25" s="2"/>
-      <c r="AL25" s="110"/>
+      <c r="AL25" s="101"/>
       <c r="AM25" s="21">
         <v>46130</v>
       </c>
@@ -2985,7 +2985,7 @@
       <c r="AP25" s="15"/>
       <c r="AQ25" s="15"/>
     </row>
-    <row r="26" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B26" s="60"/>
       <c r="C26" s="12">
         <v>46010</v>
@@ -3000,7 +3000,7 @@
         <v>7</v>
       </c>
       <c r="G26" s="2"/>
-      <c r="H26" s="110" t="s">
+      <c r="H26" s="101" t="s">
         <v>34</v>
       </c>
       <c r="I26" s="12">
@@ -3014,7 +3014,7 @@
         <v>7</v>
       </c>
       <c r="M26" s="35"/>
-      <c r="N26" s="110"/>
+      <c r="N26" s="101"/>
       <c r="O26" s="1">
         <v>46072</v>
       </c>
@@ -3022,13 +3022,13 @@
       <c r="Q26" s="3"/>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
-      <c r="T26" s="114"/>
+      <c r="T26" s="96"/>
       <c r="U26" s="71"/>
       <c r="V26" s="77"/>
       <c r="W26" s="76"/>
       <c r="X26" s="75"/>
       <c r="Y26" s="75"/>
-      <c r="Z26" s="111"/>
+      <c r="Z26" s="99"/>
       <c r="AA26" s="1">
         <v>46072</v>
       </c>
@@ -3040,7 +3040,7 @@
       <c r="AE26" s="2">
         <v>7</v>
       </c>
-      <c r="AF26" s="110"/>
+      <c r="AF26" s="101"/>
       <c r="AG26" s="12">
         <v>46100</v>
       </c>
@@ -3052,7 +3052,7 @@
         <v>7</v>
       </c>
       <c r="AK26" s="2"/>
-      <c r="AL26" s="110"/>
+      <c r="AL26" s="101"/>
       <c r="AM26" s="21">
         <v>46131</v>
       </c>
@@ -3061,7 +3061,7 @@
       <c r="AP26" s="15"/>
       <c r="AQ26" s="15"/>
     </row>
-    <row r="27" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="60"/>
       <c r="C27" s="21">
         <v>46011</v>
@@ -3070,7 +3070,7 @@
       <c r="E27" s="17"/>
       <c r="F27" s="15"/>
       <c r="G27" s="15"/>
-      <c r="H27" s="110"/>
+      <c r="H27" s="101"/>
       <c r="I27" s="12">
         <v>46042</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>7</v>
       </c>
       <c r="M27" s="35"/>
-      <c r="N27" s="110"/>
+      <c r="N27" s="101"/>
       <c r="O27" s="1">
         <v>46073</v>
       </c>
@@ -3090,13 +3090,13 @@
       <c r="Q27" s="3"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
-      <c r="T27" s="114"/>
+      <c r="T27" s="96"/>
       <c r="U27" s="71"/>
       <c r="V27" s="77"/>
       <c r="W27" s="76"/>
       <c r="X27" s="75"/>
       <c r="Y27" s="75"/>
-      <c r="Z27" s="111"/>
+      <c r="Z27" s="99"/>
       <c r="AA27" s="1">
         <v>46073</v>
       </c>
@@ -3108,7 +3108,7 @@
       <c r="AE27" s="2">
         <v>7</v>
       </c>
-      <c r="AF27" s="110"/>
+      <c r="AF27" s="101"/>
       <c r="AG27" s="12">
         <v>46101</v>
       </c>
@@ -3120,7 +3120,7 @@
         <v>7</v>
       </c>
       <c r="AK27" s="2"/>
-      <c r="AL27" s="110" t="s">
+      <c r="AL27" s="101" t="s">
         <v>35</v>
       </c>
       <c r="AM27" s="12">
@@ -3131,7 +3131,7 @@
       <c r="AP27" s="2"/>
       <c r="AQ27" s="2"/>
     </row>
-    <row r="28" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B28" s="47"/>
       <c r="C28" s="21">
         <v>46012</v>
@@ -3140,7 +3140,7 @@
       <c r="E28" s="14"/>
       <c r="F28" s="15"/>
       <c r="G28" s="15"/>
-      <c r="H28" s="110"/>
+      <c r="H28" s="101"/>
       <c r="I28" s="12">
         <v>46043</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>7</v>
       </c>
       <c r="M28" s="35"/>
-      <c r="N28" s="110"/>
+      <c r="N28" s="101"/>
       <c r="O28" s="14">
         <v>46074</v>
       </c>
@@ -3160,13 +3160,13 @@
       <c r="Q28" s="14"/>
       <c r="R28" s="15"/>
       <c r="S28" s="15"/>
-      <c r="T28" s="114"/>
+      <c r="T28" s="96"/>
       <c r="U28" s="71"/>
       <c r="V28" s="76"/>
       <c r="W28" s="76"/>
       <c r="X28" s="75"/>
       <c r="Y28" s="75"/>
-      <c r="Z28" s="111"/>
+      <c r="Z28" s="99"/>
       <c r="AA28" s="14">
         <v>46074</v>
       </c>
@@ -3174,7 +3174,7 @@
       <c r="AC28" s="14"/>
       <c r="AD28" s="15"/>
       <c r="AE28" s="15"/>
-      <c r="AF28" s="110"/>
+      <c r="AF28" s="101"/>
       <c r="AG28" s="21">
         <v>46102</v>
       </c>
@@ -3182,7 +3182,7 @@
       <c r="AI28" s="14"/>
       <c r="AJ28" s="15"/>
       <c r="AK28" s="15"/>
-      <c r="AL28" s="110"/>
+      <c r="AL28" s="101"/>
       <c r="AM28" s="12">
         <v>46133</v>
       </c>
@@ -3191,7 +3191,7 @@
       <c r="AP28" s="27"/>
       <c r="AQ28" s="27"/>
     </row>
-    <row r="29" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="46"/>
       <c r="C29" s="21">
         <v>46013</v>
@@ -3202,7 +3202,7 @@
       <c r="E29" s="49"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15"/>
-      <c r="H29" s="110"/>
+      <c r="H29" s="101"/>
       <c r="I29" s="12">
         <v>46044</v>
       </c>
@@ -3214,7 +3214,7 @@
         <v>7</v>
       </c>
       <c r="M29" s="35"/>
-      <c r="N29" s="110"/>
+      <c r="N29" s="101"/>
       <c r="O29" s="14">
         <v>46075</v>
       </c>
@@ -3222,13 +3222,13 @@
       <c r="Q29" s="14"/>
       <c r="R29" s="15"/>
       <c r="S29" s="15"/>
-      <c r="T29" s="114"/>
+      <c r="T29" s="96"/>
       <c r="U29" s="71"/>
       <c r="V29" s="76"/>
       <c r="W29" s="76"/>
       <c r="X29" s="75"/>
       <c r="Y29" s="75"/>
-      <c r="Z29" s="111"/>
+      <c r="Z29" s="99"/>
       <c r="AA29" s="14">
         <v>46075</v>
       </c>
@@ -3236,7 +3236,7 @@
       <c r="AC29" s="14"/>
       <c r="AD29" s="15"/>
       <c r="AE29" s="15"/>
-      <c r="AF29" s="110"/>
+      <c r="AF29" s="101"/>
       <c r="AG29" s="21">
         <v>46103</v>
       </c>
@@ -3244,7 +3244,7 @@
       <c r="AI29" s="14"/>
       <c r="AJ29" s="15"/>
       <c r="AK29" s="15"/>
-      <c r="AL29" s="110"/>
+      <c r="AL29" s="101"/>
       <c r="AM29" s="12">
         <v>46134</v>
       </c>
@@ -3253,7 +3253,7 @@
       <c r="AP29" s="2"/>
       <c r="AQ29" s="2"/>
     </row>
-    <row r="30" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B30" s="60"/>
       <c r="C30" s="21">
         <v>46014</v>
@@ -3262,7 +3262,7 @@
       <c r="E30" s="51"/>
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
-      <c r="H30" s="110"/>
+      <c r="H30" s="101"/>
       <c r="I30" s="12">
         <v>46045</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>7</v>
       </c>
       <c r="M30" s="35"/>
-      <c r="N30" s="110" t="s">
+      <c r="N30" s="101" t="s">
         <v>38</v>
       </c>
       <c r="O30" s="1">
@@ -3284,13 +3284,13 @@
       <c r="Q30" s="1"/>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
-      <c r="T30" s="114"/>
+      <c r="T30" s="96"/>
       <c r="U30" s="71"/>
       <c r="V30" s="76"/>
       <c r="W30" s="76"/>
       <c r="X30" s="75"/>
       <c r="Y30" s="75"/>
-      <c r="Z30" s="111" t="s">
+      <c r="Z30" s="99" t="s">
         <v>38</v>
       </c>
       <c r="AA30" s="1">
@@ -3304,7 +3304,7 @@
       <c r="AE30" s="2">
         <v>7</v>
       </c>
-      <c r="AF30" s="110" t="s">
+      <c r="AF30" s="101" t="s">
         <v>39</v>
       </c>
       <c r="AG30" s="12">
@@ -3318,7 +3318,7 @@
         <v>7</v>
       </c>
       <c r="AK30" s="2"/>
-      <c r="AL30" s="110"/>
+      <c r="AL30" s="101"/>
       <c r="AM30" s="12">
         <v>46135</v>
       </c>
@@ -3327,7 +3327,7 @@
       <c r="AP30" s="2"/>
       <c r="AQ30" s="2"/>
     </row>
-    <row r="31" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="60"/>
       <c r="C31" s="21">
         <v>46015</v>
@@ -3336,7 +3336,7 @@
       <c r="E31" s="51"/>
       <c r="F31" s="15"/>
       <c r="G31" s="15"/>
-      <c r="H31" s="110"/>
+      <c r="H31" s="101"/>
       <c r="I31" s="21">
         <v>46046</v>
       </c>
@@ -3344,7 +3344,7 @@
       <c r="K31" s="14"/>
       <c r="L31" s="15"/>
       <c r="M31" s="20"/>
-      <c r="N31" s="110"/>
+      <c r="N31" s="101"/>
       <c r="O31" s="1">
         <v>46077</v>
       </c>
@@ -3352,13 +3352,13 @@
       <c r="Q31" s="1"/>
       <c r="R31" s="2"/>
       <c r="S31" s="2"/>
-      <c r="T31" s="114"/>
+      <c r="T31" s="96"/>
       <c r="U31" s="71"/>
       <c r="V31" s="71"/>
       <c r="W31" s="71"/>
       <c r="X31" s="75"/>
       <c r="Y31" s="75"/>
-      <c r="Z31" s="111"/>
+      <c r="Z31" s="99"/>
       <c r="AA31" s="1">
         <v>46077</v>
       </c>
@@ -3370,7 +3370,7 @@
       <c r="AE31" s="2">
         <v>7</v>
       </c>
-      <c r="AF31" s="110"/>
+      <c r="AF31" s="101"/>
       <c r="AG31" s="12">
         <v>46105</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>7</v>
       </c>
       <c r="AK31" s="2"/>
-      <c r="AL31" s="110"/>
+      <c r="AL31" s="101"/>
       <c r="AM31" s="12">
         <v>46136</v>
       </c>
@@ -3391,7 +3391,7 @@
       <c r="AP31" s="2"/>
       <c r="AQ31" s="2"/>
     </row>
-    <row r="32" spans="2:43" ht="18" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:43" ht="19.5" x14ac:dyDescent="0.25">
       <c r="B32" s="60" t="s">
         <v>36</v>
       </c>
@@ -3402,7 +3402,7 @@
       <c r="E32" s="51"/>
       <c r="F32" s="15"/>
       <c r="G32" s="15"/>
-      <c r="H32" s="110"/>
+      <c r="H32" s="101"/>
       <c r="I32" s="21">
         <v>46047</v>
       </c>
@@ -3410,7 +3410,7 @@
       <c r="K32" s="17"/>
       <c r="L32" s="15"/>
       <c r="M32" s="20"/>
-      <c r="N32" s="110"/>
+      <c r="N32" s="101"/>
       <c r="O32" s="1">
         <v>46078</v>
       </c>
@@ -3418,13 +3418,13 @@
       <c r="Q32" s="1"/>
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
-      <c r="T32" s="114"/>
+      <c r="T32" s="96"/>
       <c r="U32" s="71"/>
       <c r="V32" s="76"/>
       <c r="W32" s="76"/>
       <c r="X32" s="75"/>
       <c r="Y32" s="75"/>
-      <c r="Z32" s="111"/>
+      <c r="Z32" s="99"/>
       <c r="AA32" s="1">
         <v>46078</v>
       </c>
@@ -3436,7 +3436,7 @@
       <c r="AE32" s="2">
         <v>7</v>
       </c>
-      <c r="AF32" s="110"/>
+      <c r="AF32" s="101"/>
       <c r="AG32" s="12">
         <v>46106</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>7</v>
       </c>
       <c r="AK32" s="2"/>
-      <c r="AL32" s="110"/>
+      <c r="AL32" s="101"/>
       <c r="AM32" s="21">
         <v>46137</v>
       </c>
@@ -3457,7 +3457,7 @@
       <c r="AP32" s="15"/>
       <c r="AQ32" s="15"/>
     </row>
-    <row r="33" spans="2:43" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:43" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="60"/>
       <c r="C33" s="21">
         <v>46017</v>
@@ -3466,7 +3466,7 @@
       <c r="E33" s="53"/>
       <c r="F33" s="18"/>
       <c r="G33" s="18"/>
-      <c r="H33" s="107" t="s">
+      <c r="H33" s="105" t="s">
         <v>40</v>
       </c>
       <c r="I33" s="12">
@@ -3482,7 +3482,7 @@
         <v>7</v>
       </c>
       <c r="M33" s="2"/>
-      <c r="N33" s="110"/>
+      <c r="N33" s="101"/>
       <c r="O33" s="1">
         <v>46079</v>
       </c>
@@ -3490,13 +3490,13 @@
       <c r="Q33" s="4"/>
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
-      <c r="T33" s="114"/>
+      <c r="T33" s="96"/>
       <c r="U33" s="71"/>
       <c r="V33" s="76"/>
       <c r="W33" s="76"/>
       <c r="X33" s="75"/>
       <c r="Y33" s="75"/>
-      <c r="Z33" s="111"/>
+      <c r="Z33" s="99"/>
       <c r="AA33" s="1">
         <v>46079</v>
       </c>
@@ -3508,7 +3508,7 @@
       <c r="AE33" s="2">
         <v>7</v>
       </c>
-      <c r="AF33" s="110"/>
+      <c r="AF33" s="101"/>
       <c r="AG33" s="12">
         <v>46107</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>7</v>
       </c>
       <c r="AK33" s="4"/>
-      <c r="AL33" s="110"/>
+      <c r="AL33" s="101"/>
       <c r="AM33" s="21">
         <v>46138</v>
       </c>
@@ -3531,7 +3531,7 @@
       <c r="AP33" s="18"/>
       <c r="AQ33" s="18"/>
     </row>
-    <row r="34" spans="2:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:43" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="60"/>
       <c r="C34" s="21">
         <v>46018</v>
@@ -3540,7 +3540,7 @@
       <c r="E34" s="14"/>
       <c r="F34" s="15"/>
       <c r="G34" s="15"/>
-      <c r="H34" s="118"/>
+      <c r="H34" s="106"/>
       <c r="I34" s="12">
         <v>46049</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>7</v>
       </c>
       <c r="M34" s="2"/>
-      <c r="N34" s="110"/>
+      <c r="N34" s="101"/>
       <c r="O34" s="1">
         <v>46080</v>
       </c>
@@ -3562,13 +3562,13 @@
       <c r="Q34" s="1"/>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
-      <c r="T34" s="114"/>
+      <c r="T34" s="96"/>
       <c r="U34" s="71"/>
       <c r="V34" s="76"/>
       <c r="W34" s="76"/>
       <c r="X34" s="75"/>
       <c r="Y34" s="75"/>
-      <c r="Z34" s="111"/>
+      <c r="Z34" s="99"/>
       <c r="AA34" s="1">
         <v>46080</v>
       </c>
@@ -3580,7 +3580,7 @@
       <c r="AE34" s="2">
         <v>7</v>
       </c>
-      <c r="AF34" s="110"/>
+      <c r="AF34" s="101"/>
       <c r="AG34" s="12">
         <v>46108</v>
       </c>
@@ -3594,7 +3594,7 @@
         <v>7</v>
       </c>
       <c r="AK34" s="2"/>
-      <c r="AL34" s="110" t="s">
+      <c r="AL34" s="101" t="s">
         <v>41</v>
       </c>
       <c r="AM34" s="12">
@@ -3605,7 +3605,7 @@
       <c r="AP34" s="2"/>
       <c r="AQ34" s="2"/>
     </row>
-    <row r="35" spans="2:43" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:43" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="47"/>
       <c r="C35" s="21">
         <v>46019</v>
@@ -3614,7 +3614,7 @@
       <c r="E35" s="14"/>
       <c r="F35" s="15"/>
       <c r="G35" s="15"/>
-      <c r="H35" s="118"/>
+      <c r="H35" s="106"/>
       <c r="I35" s="12">
         <v>46050</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>7</v>
       </c>
       <c r="M35" s="2"/>
-      <c r="N35" s="110"/>
+      <c r="N35" s="101"/>
       <c r="O35" s="14">
         <v>46081</v>
       </c>
@@ -3636,13 +3636,13 @@
       <c r="Q35" s="14"/>
       <c r="R35" s="15"/>
       <c r="S35" s="15"/>
-      <c r="T35" s="114"/>
+      <c r="T35" s="96"/>
       <c r="U35" s="71"/>
       <c r="V35" s="76"/>
       <c r="W35" s="76"/>
       <c r="X35" s="75"/>
       <c r="Y35" s="75"/>
-      <c r="Z35" s="111"/>
+      <c r="Z35" s="99"/>
       <c r="AA35" s="14">
         <v>46081</v>
       </c>
@@ -3650,7 +3650,7 @@
       <c r="AC35" s="14"/>
       <c r="AD35" s="15"/>
       <c r="AE35" s="15"/>
-      <c r="AF35" s="110"/>
+      <c r="AF35" s="101"/>
       <c r="AG35" s="21">
         <v>46109</v>
       </c>
@@ -3658,7 +3658,7 @@
       <c r="AI35" s="14"/>
       <c r="AJ35" s="15"/>
       <c r="AK35" s="15"/>
-      <c r="AL35" s="110"/>
+      <c r="AL35" s="101"/>
       <c r="AM35" s="12">
         <v>46140</v>
       </c>
@@ -3667,7 +3667,7 @@
       <c r="AP35" s="2"/>
       <c r="AQ35" s="2"/>
     </row>
-    <row r="36" spans="2:43" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:43" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="46"/>
       <c r="C36" s="21">
         <v>46020</v>
@@ -3678,7 +3678,7 @@
       <c r="E36" s="55"/>
       <c r="F36" s="19"/>
       <c r="G36" s="19"/>
-      <c r="H36" s="118"/>
+      <c r="H36" s="106"/>
       <c r="I36" s="12">
         <v>46051</v>
       </c>
@@ -3692,25 +3692,25 @@
         <v>7</v>
       </c>
       <c r="M36" s="2"/>
-      <c r="N36" s="110"/>
-      <c r="O36" s="110"/>
-      <c r="P36" s="110"/>
-      <c r="Q36" s="110"/>
-      <c r="R36" s="110"/>
-      <c r="S36" s="110"/>
-      <c r="T36" s="114"/>
+      <c r="N36" s="101"/>
+      <c r="O36" s="101"/>
+      <c r="P36" s="101"/>
+      <c r="Q36" s="101"/>
+      <c r="R36" s="101"/>
+      <c r="S36" s="101"/>
+      <c r="T36" s="96"/>
       <c r="U36" s="71"/>
       <c r="V36" s="3"/>
       <c r="W36" s="76"/>
       <c r="X36" s="75"/>
       <c r="Y36" s="75"/>
-      <c r="Z36" s="111"/>
-      <c r="AA36" s="110"/>
-      <c r="AB36" s="110"/>
-      <c r="AC36" s="110"/>
-      <c r="AD36" s="110"/>
-      <c r="AE36" s="110"/>
-      <c r="AF36" s="110"/>
+      <c r="Z36" s="99"/>
+      <c r="AA36" s="101"/>
+      <c r="AB36" s="101"/>
+      <c r="AC36" s="101"/>
+      <c r="AD36" s="101"/>
+      <c r="AE36" s="101"/>
+      <c r="AF36" s="101"/>
       <c r="AG36" s="21">
         <v>46110</v>
       </c>
@@ -3718,7 +3718,7 @@
       <c r="AI36" s="19"/>
       <c r="AJ36" s="19"/>
       <c r="AK36" s="19"/>
-      <c r="AL36" s="110"/>
+      <c r="AL36" s="101"/>
       <c r="AM36" s="12">
         <v>46141</v>
       </c>
@@ -3727,7 +3727,7 @@
       <c r="AP36" s="8"/>
       <c r="AQ36" s="8"/>
     </row>
-    <row r="37" spans="2:43" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:43" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="60"/>
       <c r="C37" s="21">
         <v>46021</v>
@@ -3736,7 +3736,7 @@
       <c r="E37" s="57"/>
       <c r="F37" s="19"/>
       <c r="G37" s="19"/>
-      <c r="H37" s="118"/>
+      <c r="H37" s="106"/>
       <c r="I37" s="12">
         <v>46052</v>
       </c>
@@ -3750,25 +3750,25 @@
         <v>7</v>
       </c>
       <c r="M37" s="2"/>
-      <c r="N37" s="110"/>
-      <c r="O37" s="110"/>
-      <c r="P37" s="110"/>
-      <c r="Q37" s="110"/>
-      <c r="R37" s="110"/>
-      <c r="S37" s="110"/>
-      <c r="T37" s="114"/>
+      <c r="N37" s="101"/>
+      <c r="O37" s="101"/>
+      <c r="P37" s="101"/>
+      <c r="Q37" s="101"/>
+      <c r="R37" s="101"/>
+      <c r="S37" s="101"/>
+      <c r="T37" s="96"/>
       <c r="U37" s="71"/>
       <c r="V37" s="76"/>
       <c r="W37" s="71"/>
       <c r="X37" s="75"/>
       <c r="Y37" s="75"/>
-      <c r="Z37" s="111"/>
-      <c r="AA37" s="110"/>
-      <c r="AB37" s="110"/>
-      <c r="AC37" s="110"/>
-      <c r="AD37" s="110"/>
-      <c r="AE37" s="110"/>
-      <c r="AF37" s="107"/>
+      <c r="Z37" s="99"/>
+      <c r="AA37" s="101"/>
+      <c r="AB37" s="101"/>
+      <c r="AC37" s="101"/>
+      <c r="AD37" s="101"/>
+      <c r="AE37" s="101"/>
+      <c r="AF37" s="105"/>
       <c r="AG37" s="12">
         <v>46111</v>
       </c>
@@ -3780,7 +3780,7 @@
         <v>7</v>
       </c>
       <c r="AK37" s="8"/>
-      <c r="AL37" s="110"/>
+      <c r="AL37" s="101"/>
       <c r="AM37" s="12">
         <v>46142</v>
       </c>
@@ -3789,7 +3789,7 @@
       <c r="AP37" s="8"/>
       <c r="AQ37" s="8"/>
     </row>
-    <row r="38" spans="2:43" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:43" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="47"/>
       <c r="C38" s="21">
         <v>46022</v>
@@ -3798,7 +3798,7 @@
       <c r="E38" s="59"/>
       <c r="F38" s="19"/>
       <c r="G38" s="19"/>
-      <c r="H38" s="108"/>
+      <c r="H38" s="107"/>
       <c r="I38" s="21">
         <v>46053</v>
       </c>
@@ -3806,25 +3806,25 @@
       <c r="K38" s="37"/>
       <c r="L38" s="38"/>
       <c r="M38" s="38"/>
-      <c r="N38" s="110"/>
-      <c r="O38" s="110"/>
-      <c r="P38" s="110"/>
-      <c r="Q38" s="110"/>
-      <c r="R38" s="110"/>
-      <c r="S38" s="110"/>
-      <c r="T38" s="114"/>
+      <c r="N38" s="101"/>
+      <c r="O38" s="101"/>
+      <c r="P38" s="101"/>
+      <c r="Q38" s="101"/>
+      <c r="R38" s="101"/>
+      <c r="S38" s="101"/>
+      <c r="T38" s="96"/>
       <c r="U38" s="71"/>
       <c r="V38" s="78"/>
       <c r="W38" s="78"/>
       <c r="X38" s="79"/>
       <c r="Y38" s="79"/>
-      <c r="Z38" s="111"/>
-      <c r="AA38" s="110"/>
-      <c r="AB38" s="110"/>
-      <c r="AC38" s="110"/>
-      <c r="AD38" s="110"/>
-      <c r="AE38" s="110"/>
-      <c r="AF38" s="108"/>
+      <c r="Z38" s="99"/>
+      <c r="AA38" s="101"/>
+      <c r="AB38" s="101"/>
+      <c r="AC38" s="101"/>
+      <c r="AD38" s="101"/>
+      <c r="AE38" s="101"/>
+      <c r="AF38" s="107"/>
       <c r="AG38" s="1">
         <v>46112</v>
       </c>
@@ -3836,14 +3836,14 @@
         <v>7</v>
       </c>
       <c r="AK38" s="8"/>
-      <c r="AL38" s="119"/>
-      <c r="AM38" s="120"/>
-      <c r="AN38" s="120"/>
-      <c r="AO38" s="120"/>
-      <c r="AP38" s="120"/>
-      <c r="AQ38" s="111"/>
-    </row>
-    <row r="39" spans="2:43" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AL38" s="97"/>
+      <c r="AM38" s="98"/>
+      <c r="AN38" s="98"/>
+      <c r="AO38" s="98"/>
+      <c r="AP38" s="98"/>
+      <c r="AQ38" s="99"/>
+    </row>
+    <row r="39" spans="2:43" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
       <c r="D39" s="11"/>
@@ -3911,7 +3911,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:43" x14ac:dyDescent="0.25">
       <c r="F40" s="5">
         <f>SUM(F8:F38)</f>
         <v>35</v>
@@ -3975,112 +3975,95 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:43" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:43" x14ac:dyDescent="0.25">
       <c r="D41" s="89" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="42" spans="2:43" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:43" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D42" s="88" t="s">
         <v>58</v>
       </c>
-      <c r="J42" s="101" t="s">
+      <c r="J42" s="108" t="s">
         <v>47</v>
       </c>
-      <c r="K42" s="102"/>
-      <c r="P42" s="97" t="s">
+      <c r="K42" s="109"/>
+      <c r="P42" s="119" t="s">
         <v>72</v>
       </c>
-      <c r="Q42" s="98"/>
-    </row>
-    <row r="43" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q42" s="120"/>
+    </row>
+    <row r="43" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D43" s="90" t="s">
         <v>59</v>
       </c>
-      <c r="J43" s="103"/>
-      <c r="K43" s="104"/>
-      <c r="P43" s="99" t="s">
+      <c r="J43" s="110"/>
+      <c r="K43" s="111"/>
+      <c r="P43" s="121" t="s">
         <v>79</v>
       </c>
-      <c r="Q43" s="100"/>
-    </row>
-    <row r="44" spans="2:43" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q43" s="122"/>
+    </row>
+    <row r="44" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D44" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="J44" s="105"/>
-      <c r="K44" s="106"/>
-      <c r="P44" s="99" t="s">
+      <c r="J44" s="112"/>
+      <c r="K44" s="113"/>
+      <c r="P44" s="121" t="s">
         <v>73</v>
       </c>
-      <c r="Q44" s="100"/>
-    </row>
-    <row r="45" spans="2:43" x14ac:dyDescent="0.3">
+      <c r="Q44" s="122"/>
+    </row>
+    <row r="45" spans="2:43" x14ac:dyDescent="0.25">
       <c r="D45" s="91" t="s">
         <v>61</v>
       </c>
-      <c r="P45" s="99" t="s">
+      <c r="P45" s="121" t="s">
         <v>74</v>
       </c>
-      <c r="Q45" s="100"/>
-    </row>
-    <row r="46" spans="2:43" x14ac:dyDescent="0.3">
-      <c r="P46" s="99" t="s">
+      <c r="Q45" s="122"/>
+    </row>
+    <row r="46" spans="2:43" x14ac:dyDescent="0.25">
+      <c r="P46" s="121" t="s">
         <v>75</v>
       </c>
-      <c r="Q46" s="100"/>
-    </row>
-    <row r="47" spans="2:43" x14ac:dyDescent="0.3">
-      <c r="D47" s="122" t="s">
+      <c r="Q46" s="122"/>
+    </row>
+    <row r="47" spans="2:43" x14ac:dyDescent="0.25">
+      <c r="D47" s="95" t="s">
         <v>80</v>
       </c>
-      <c r="P47" s="99" t="s">
+      <c r="P47" s="121" t="s">
         <v>76</v>
       </c>
-      <c r="Q47" s="100"/>
-    </row>
-    <row r="48" spans="2:43" x14ac:dyDescent="0.3">
-      <c r="D48" s="122" t="s">
+      <c r="Q47" s="122"/>
+    </row>
+    <row r="48" spans="2:43" x14ac:dyDescent="0.25">
+      <c r="D48" s="95" t="s">
         <v>81</v>
       </c>
-      <c r="P48" s="95" t="s">
+      <c r="P48" s="117" t="s">
         <v>77</v>
       </c>
-      <c r="Q48" s="96"/>
-    </row>
-    <row r="49" spans="16:17" x14ac:dyDescent="0.3">
-      <c r="P49" s="95" t="s">
+      <c r="Q48" s="118"/>
+    </row>
+    <row r="49" spans="16:17" x14ac:dyDescent="0.25">
+      <c r="P49" s="117" t="s">
         <v>78</v>
       </c>
-      <c r="Q49" s="96"/>
+      <c r="Q49" s="118"/>
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="T8:T11"/>
-    <mergeCell ref="AL38:AQ38"/>
-    <mergeCell ref="AL6:AQ6"/>
-    <mergeCell ref="AL8:AL12"/>
-    <mergeCell ref="AL13:AL19"/>
-    <mergeCell ref="AN13:AO13"/>
-    <mergeCell ref="AL20:AL26"/>
-    <mergeCell ref="AL27:AL33"/>
-    <mergeCell ref="AL34:AL37"/>
-    <mergeCell ref="T19:T25"/>
-    <mergeCell ref="Z23:Z29"/>
-    <mergeCell ref="T26:T32"/>
-    <mergeCell ref="Z30:Z35"/>
-    <mergeCell ref="Z16:Z22"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="N9:N15"/>
-    <mergeCell ref="H12:H18"/>
-    <mergeCell ref="N16:N22"/>
-    <mergeCell ref="H19:H25"/>
-    <mergeCell ref="N23:N29"/>
-    <mergeCell ref="H26:H32"/>
-    <mergeCell ref="N30:N35"/>
-    <mergeCell ref="H33:H38"/>
-    <mergeCell ref="N36:S38"/>
+    <mergeCell ref="P48:Q48"/>
+    <mergeCell ref="P49:Q49"/>
+    <mergeCell ref="P42:Q42"/>
+    <mergeCell ref="P44:Q44"/>
+    <mergeCell ref="P45:Q45"/>
+    <mergeCell ref="P46:Q46"/>
+    <mergeCell ref="P47:Q47"/>
+    <mergeCell ref="P43:Q43"/>
     <mergeCell ref="J42:K44"/>
     <mergeCell ref="AF37:AF38"/>
     <mergeCell ref="AF6:AK6"/>
@@ -4097,14 +4080,31 @@
     <mergeCell ref="Z9:Z15"/>
     <mergeCell ref="T12:T18"/>
     <mergeCell ref="H6:M6"/>
-    <mergeCell ref="P48:Q48"/>
-    <mergeCell ref="P49:Q49"/>
-    <mergeCell ref="P42:Q42"/>
-    <mergeCell ref="P44:Q44"/>
-    <mergeCell ref="P45:Q45"/>
-    <mergeCell ref="P46:Q46"/>
-    <mergeCell ref="P47:Q47"/>
-    <mergeCell ref="P43:Q43"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="N9:N15"/>
+    <mergeCell ref="H12:H18"/>
+    <mergeCell ref="N16:N22"/>
+    <mergeCell ref="H19:H25"/>
+    <mergeCell ref="N23:N29"/>
+    <mergeCell ref="H26:H32"/>
+    <mergeCell ref="N30:N35"/>
+    <mergeCell ref="H33:H38"/>
+    <mergeCell ref="N36:S38"/>
+    <mergeCell ref="T8:T11"/>
+    <mergeCell ref="AL38:AQ38"/>
+    <mergeCell ref="AL6:AQ6"/>
+    <mergeCell ref="AL8:AL12"/>
+    <mergeCell ref="AL13:AL19"/>
+    <mergeCell ref="AN13:AO13"/>
+    <mergeCell ref="AL20:AL26"/>
+    <mergeCell ref="AL27:AL33"/>
+    <mergeCell ref="AL34:AL37"/>
+    <mergeCell ref="T19:T25"/>
+    <mergeCell ref="Z23:Z29"/>
+    <mergeCell ref="T26:T32"/>
+    <mergeCell ref="Z30:Z35"/>
+    <mergeCell ref="Z16:Z22"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4124,15 +4124,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100862694ECED4E1948B5E8D6F6BADC8D0D" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="ae739b22c1d0ad2d0a68cf71a23d442c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="102bceca-7b01-449b-a089-7caeaaf28d79" xmlns:ns3="7fc2edd5-909c-43a2-b3b4-2537dcd3eee1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="05a22d24dcf35b0ff3f755cd1ef480a8" ns2:_="" ns3:_="">
     <xsd:import namespace="102bceca-7b01-449b-a089-7caeaaf28d79"/>
@@ -4333,6 +4324,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{027A5389-2971-44C0-A0D1-6195B9A552F9}">
   <ds:schemaRefs>
@@ -4351,14 +4351,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23969816-9B9E-4320-B349-9EB0D8911C7F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4F02508-5572-4BFA-B015-F122D6CC4035}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4375,4 +4367,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23969816-9B9E-4320-B349-9EB0D8911C7F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: Add logistics training documents and planning spreadsheets.
</commit_message>
<xml_diff>
--- a/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/Planning prévisionnel Habilitations Nucléaires 3 Ok.xlsx
+++ b/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/Planning prévisionnel Habilitations Nucléaires 3 Ok.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E929FCC-ACDD-47E0-A12F-F4FC7BA36476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D17A5247-4B7E-4F2D-8051-B78F30B21410}"/>
+    <workbookView minimized="1" xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{D17A5247-4B7E-4F2D-8051-B78F30B21410}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -4113,6 +4113,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="102bceca-7b01-449b-a089-7caeaaf28d79">
@@ -4123,7 +4132,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100862694ECED4E1948B5E8D6F6BADC8D0D" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="ae739b22c1d0ad2d0a68cf71a23d442c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="102bceca-7b01-449b-a089-7caeaaf28d79" xmlns:ns3="7fc2edd5-909c-43a2-b3b4-2537dcd3eee1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="05a22d24dcf35b0ff3f755cd1ef480a8" ns2:_="" ns3:_="">
     <xsd:import namespace="102bceca-7b01-449b-a089-7caeaaf28d79"/>
@@ -4324,16 +4333,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23969816-9B9E-4320-B349-9EB0D8911C7F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{027A5389-2971-44C0-A0D1-6195B9A552F9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -4350,7 +4358,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4F02508-5572-4BFA-B015-F122D6CC4035}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4367,12 +4375,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23969816-9B9E-4320-B349-9EB0D8911C7F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore: delete a file from the repository
</commit_message>
<xml_diff>
--- a/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/Planning prévisionnel Habilitations Nucléaires 3 Ok.xlsx
+++ b/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/Planning prévisionnel Habilitations Nucléaires 3 Ok.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E929FCC-ACDD-47E0-A12F-F4FC7BA36476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{D17A5247-4B7E-4F2D-8051-B78F30B21410}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D17A5247-4B7E-4F2D-8051-B78F30B21410}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -4113,15 +4113,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="102bceca-7b01-449b-a089-7caeaaf28d79">
@@ -4132,7 +4123,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100862694ECED4E1948B5E8D6F6BADC8D0D" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="ae739b22c1d0ad2d0a68cf71a23d442c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="102bceca-7b01-449b-a089-7caeaaf28d79" xmlns:ns3="7fc2edd5-909c-43a2-b3b4-2537dcd3eee1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="05a22d24dcf35b0ff3f755cd1ef480a8" ns2:_="" ns3:_="">
     <xsd:import namespace="102bceca-7b01-449b-a089-7caeaaf28d79"/>
@@ -4333,15 +4324,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23969816-9B9E-4320-B349-9EB0D8911C7F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{027A5389-2971-44C0-A0D1-6195B9A552F9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -4358,7 +4350,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4F02508-5572-4BFA-B015-F122D6CC4035}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4375,4 +4367,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23969816-9B9E-4320-B349-9EB0D8911C7F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor: improve textarea auto-resize and scrollbar behavior in chat input.
</commit_message>
<xml_diff>
--- a/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/Planning prévisionnel Habilitations Nucléaires 3 Ok.xlsx
+++ b/OI/Habilitations Nucléaires Ouzouer sur Loire 28-29 Janv 9-10-11 Fev/Planning prévisionnel Habilitations Nucléaires 3 Ok.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E929FCC-ACDD-47E0-A12F-F4FC7BA36476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="30" windowWidth="28770" windowHeight="15450" xr2:uid="{D17A5247-4B7E-4F2D-8051-B78F30B21410}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{D17A5247-4B7E-4F2D-8051-B78F30B21410}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -1041,6 +1041,69 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1058,69 +1121,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1548,52 +1548,52 @@
       <c r="E6" s="63"/>
       <c r="F6" s="63"/>
       <c r="G6" s="61"/>
-      <c r="H6" s="110" t="s">
+      <c r="H6" s="100" t="s">
         <v>3</v>
       </c>
-      <c r="I6" s="110"/>
-      <c r="J6" s="110"/>
-      <c r="K6" s="110"/>
-      <c r="L6" s="110"/>
-      <c r="M6" s="110"/>
-      <c r="N6" s="110" t="s">
+      <c r="I6" s="100"/>
+      <c r="J6" s="100"/>
+      <c r="K6" s="100"/>
+      <c r="L6" s="100"/>
+      <c r="M6" s="100"/>
+      <c r="N6" s="100" t="s">
         <v>4</v>
       </c>
-      <c r="O6" s="110"/>
-      <c r="P6" s="110"/>
-      <c r="Q6" s="110"/>
-      <c r="R6" s="110"/>
-      <c r="S6" s="110"/>
-      <c r="T6" s="114"/>
-      <c r="U6" s="114"/>
-      <c r="V6" s="114"/>
-      <c r="W6" s="114"/>
-      <c r="X6" s="114"/>
-      <c r="Y6" s="114"/>
+      <c r="O6" s="100"/>
+      <c r="P6" s="100"/>
+      <c r="Q6" s="100"/>
+      <c r="R6" s="100"/>
+      <c r="S6" s="100"/>
+      <c r="T6" s="115"/>
+      <c r="U6" s="115"/>
+      <c r="V6" s="115"/>
+      <c r="W6" s="115"/>
+      <c r="X6" s="115"/>
+      <c r="Y6" s="115"/>
       <c r="Z6" s="116" t="s">
         <v>4</v>
       </c>
-      <c r="AA6" s="110"/>
-      <c r="AB6" s="110"/>
-      <c r="AC6" s="110"/>
-      <c r="AD6" s="110"/>
-      <c r="AE6" s="110"/>
-      <c r="AF6" s="110" t="s">
+      <c r="AA6" s="100"/>
+      <c r="AB6" s="100"/>
+      <c r="AC6" s="100"/>
+      <c r="AD6" s="100"/>
+      <c r="AE6" s="100"/>
+      <c r="AF6" s="100" t="s">
         <v>5</v>
       </c>
-      <c r="AG6" s="110"/>
-      <c r="AH6" s="110"/>
-      <c r="AI6" s="110"/>
-      <c r="AJ6" s="110"/>
-      <c r="AK6" s="110"/>
-      <c r="AL6" s="110" t="s">
+      <c r="AG6" s="100"/>
+      <c r="AH6" s="100"/>
+      <c r="AI6" s="100"/>
+      <c r="AJ6" s="100"/>
+      <c r="AK6" s="100"/>
+      <c r="AL6" s="100" t="s">
         <v>6</v>
       </c>
-      <c r="AM6" s="110"/>
-      <c r="AN6" s="110"/>
-      <c r="AO6" s="110"/>
-      <c r="AP6" s="110"/>
-      <c r="AQ6" s="110"/>
+      <c r="AM6" s="100"/>
+      <c r="AN6" s="100"/>
+      <c r="AO6" s="100"/>
+      <c r="AP6" s="100"/>
+      <c r="AQ6" s="100"/>
     </row>
     <row r="7" spans="2:43" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="13"/>
@@ -1696,16 +1696,16 @@
       <c r="E8" s="28"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="111" t="s">
+      <c r="H8" s="101" t="s">
         <v>14</v>
       </c>
       <c r="I8" s="21">
         <v>46023</v>
       </c>
-      <c r="J8" s="117" t="s">
+      <c r="J8" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="118"/>
+      <c r="K8" s="104"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
       <c r="N8" s="8"/>
@@ -1716,10 +1716,10 @@
       <c r="Q8" s="14"/>
       <c r="R8" s="15"/>
       <c r="S8" s="15"/>
-      <c r="T8" s="115"/>
+      <c r="T8" s="96"/>
       <c r="U8" s="71"/>
-      <c r="V8" s="113"/>
-      <c r="W8" s="113"/>
+      <c r="V8" s="114"/>
+      <c r="W8" s="114"/>
       <c r="X8" s="73"/>
       <c r="Y8" s="73"/>
       <c r="Z8" s="66"/>
@@ -1738,7 +1738,7 @@
       <c r="AI8" s="14"/>
       <c r="AJ8" s="15"/>
       <c r="AK8" s="15"/>
-      <c r="AL8" s="111" t="s">
+      <c r="AL8" s="101" t="s">
         <v>15</v>
       </c>
       <c r="AM8" s="12">
@@ -1762,7 +1762,7 @@
       <c r="E9" s="29"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="111"/>
+      <c r="H9" s="101"/>
       <c r="I9" s="21">
         <v>46024</v>
       </c>
@@ -1770,7 +1770,7 @@
       <c r="K9" s="14"/>
       <c r="L9" s="33"/>
       <c r="M9" s="34"/>
-      <c r="N9" s="111" t="s">
+      <c r="N9" s="101" t="s">
         <v>16</v>
       </c>
       <c r="O9" s="1">
@@ -1786,13 +1786,13 @@
         <v>7</v>
       </c>
       <c r="S9" s="2"/>
-      <c r="T9" s="115"/>
+      <c r="T9" s="96"/>
       <c r="U9" s="71"/>
       <c r="V9" s="71"/>
       <c r="W9" s="71"/>
       <c r="X9" s="74"/>
       <c r="Y9" s="74"/>
-      <c r="Z9" s="112" t="s">
+      <c r="Z9" s="99" t="s">
         <v>16</v>
       </c>
       <c r="AA9" s="1">
@@ -1806,7 +1806,7 @@
         <v>7</v>
       </c>
       <c r="AE9" s="2"/>
-      <c r="AF9" s="111" t="s">
+      <c r="AF9" s="101" t="s">
         <v>17</v>
       </c>
       <c r="AG9" s="12">
@@ -1820,7 +1820,7 @@
       <c r="AK9" s="2">
         <v>7</v>
       </c>
-      <c r="AL9" s="111"/>
+      <c r="AL9" s="101"/>
       <c r="AM9" s="12">
         <v>46114</v>
       </c>
@@ -1842,7 +1842,7 @@
       <c r="E10" s="29"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
-      <c r="H10" s="111"/>
+      <c r="H10" s="101"/>
       <c r="I10" s="21">
         <v>46025</v>
       </c>
@@ -1850,7 +1850,7 @@
       <c r="K10" s="14"/>
       <c r="L10" s="15"/>
       <c r="M10" s="20"/>
-      <c r="N10" s="111"/>
+      <c r="N10" s="101"/>
       <c r="O10" s="1">
         <v>46056</v>
       </c>
@@ -1864,13 +1864,13 @@
         <v>7</v>
       </c>
       <c r="S10" s="2"/>
-      <c r="T10" s="115"/>
+      <c r="T10" s="96"/>
       <c r="U10" s="71"/>
       <c r="V10" s="71"/>
       <c r="W10" s="71"/>
       <c r="X10" s="75"/>
       <c r="Y10" s="75"/>
-      <c r="Z10" s="112"/>
+      <c r="Z10" s="99"/>
       <c r="AA10" s="1">
         <v>46056</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>7</v>
       </c>
       <c r="AE10" s="2"/>
-      <c r="AF10" s="111"/>
+      <c r="AF10" s="101"/>
       <c r="AG10" s="12">
         <v>46084</v>
       </c>
@@ -1894,7 +1894,7 @@
       <c r="AK10" s="2">
         <v>7</v>
       </c>
-      <c r="AL10" s="111"/>
+      <c r="AL10" s="101"/>
       <c r="AM10" s="12">
         <v>46115</v>
       </c>
@@ -1918,7 +1918,7 @@
       <c r="E11" s="29"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="111"/>
+      <c r="H11" s="101"/>
       <c r="I11" s="21">
         <v>46026</v>
       </c>
@@ -1926,7 +1926,7 @@
       <c r="K11" s="14"/>
       <c r="L11" s="15"/>
       <c r="M11" s="20"/>
-      <c r="N11" s="111"/>
+      <c r="N11" s="101"/>
       <c r="O11" s="1">
         <v>46057</v>
       </c>
@@ -1940,13 +1940,13 @@
         <v>7</v>
       </c>
       <c r="S11" s="2"/>
-      <c r="T11" s="115"/>
+      <c r="T11" s="96"/>
       <c r="U11" s="71"/>
       <c r="V11" s="71"/>
       <c r="W11" s="71"/>
       <c r="X11" s="75"/>
       <c r="Y11" s="75"/>
-      <c r="Z11" s="112"/>
+      <c r="Z11" s="99"/>
       <c r="AA11" s="1">
         <v>46057</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>7</v>
       </c>
       <c r="AE11" s="2"/>
-      <c r="AF11" s="111"/>
+      <c r="AF11" s="101"/>
       <c r="AG11" s="12">
         <v>46085</v>
       </c>
@@ -1970,7 +1970,7 @@
       <c r="AK11" s="2">
         <v>7</v>
       </c>
-      <c r="AL11" s="111"/>
+      <c r="AL11" s="101"/>
       <c r="AM11" s="21">
         <v>46116</v>
       </c>
@@ -1988,7 +1988,7 @@
       <c r="E12" s="29"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="111" t="s">
+      <c r="H12" s="101" t="s">
         <v>18</v>
       </c>
       <c r="I12" s="12">
@@ -2004,7 +2004,7 @@
         <v>7</v>
       </c>
       <c r="M12" s="2"/>
-      <c r="N12" s="111"/>
+      <c r="N12" s="101"/>
       <c r="O12" s="1">
         <v>46058</v>
       </c>
@@ -2018,13 +2018,13 @@
         <v>7</v>
       </c>
       <c r="S12" s="2"/>
-      <c r="T12" s="115"/>
+      <c r="T12" s="96"/>
       <c r="U12" s="71"/>
       <c r="V12" s="76"/>
       <c r="W12" s="71"/>
       <c r="X12" s="75"/>
       <c r="Y12" s="75"/>
-      <c r="Z12" s="112"/>
+      <c r="Z12" s="99"/>
       <c r="AA12" s="1">
         <v>46058</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>7</v>
       </c>
       <c r="AE12" s="2"/>
-      <c r="AF12" s="111"/>
+      <c r="AF12" s="101"/>
       <c r="AG12" s="12">
         <v>46086</v>
       </c>
@@ -2048,7 +2048,7 @@
       <c r="AK12" s="2">
         <v>7</v>
       </c>
-      <c r="AL12" s="111"/>
+      <c r="AL12" s="101"/>
       <c r="AM12" s="21">
         <v>46117</v>
       </c>
@@ -2066,7 +2066,7 @@
       <c r="E13" s="30"/>
       <c r="F13" s="15"/>
       <c r="G13" s="15"/>
-      <c r="H13" s="111"/>
+      <c r="H13" s="101"/>
       <c r="I13" s="12">
         <v>46028</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>7</v>
       </c>
       <c r="M13" s="2"/>
-      <c r="N13" s="111"/>
+      <c r="N13" s="101"/>
       <c r="O13" s="1">
         <v>46059</v>
       </c>
@@ -2092,13 +2092,13 @@
         <v>7</v>
       </c>
       <c r="S13" s="2"/>
-      <c r="T13" s="115"/>
+      <c r="T13" s="96"/>
       <c r="U13" s="71"/>
       <c r="V13" s="76"/>
       <c r="W13" s="71"/>
       <c r="X13" s="75"/>
       <c r="Y13" s="75"/>
-      <c r="Z13" s="112"/>
+      <c r="Z13" s="99"/>
       <c r="AA13" s="1">
         <v>46059</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>7</v>
       </c>
       <c r="AE13" s="2"/>
-      <c r="AF13" s="111"/>
+      <c r="AF13" s="101"/>
       <c r="AG13" s="12">
         <v>46087</v>
       </c>
@@ -2122,16 +2122,16 @@
       <c r="AK13" s="2">
         <v>7</v>
       </c>
-      <c r="AL13" s="111" t="s">
+      <c r="AL13" s="101" t="s">
         <v>21</v>
       </c>
       <c r="AM13" s="21">
         <v>46118</v>
       </c>
-      <c r="AN13" s="117" t="s">
+      <c r="AN13" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="AO13" s="122"/>
+      <c r="AO13" s="103"/>
       <c r="AP13" s="15"/>
       <c r="AQ13" s="15"/>
     </row>
@@ -2144,7 +2144,7 @@
       <c r="E14" s="21"/>
       <c r="F14" s="15"/>
       <c r="G14" s="15"/>
-      <c r="H14" s="111"/>
+      <c r="H14" s="101"/>
       <c r="I14" s="12">
         <v>46029</v>
       </c>
@@ -2156,7 +2156,7 @@
         <v>7</v>
       </c>
       <c r="M14" s="2"/>
-      <c r="N14" s="111"/>
+      <c r="N14" s="101"/>
       <c r="O14" s="14">
         <v>46060</v>
       </c>
@@ -2164,13 +2164,13 @@
       <c r="Q14" s="14"/>
       <c r="R14" s="15"/>
       <c r="S14" s="15"/>
-      <c r="T14" s="115"/>
+      <c r="T14" s="96"/>
       <c r="U14" s="71"/>
       <c r="V14" s="76"/>
       <c r="W14" s="71"/>
       <c r="X14" s="75"/>
       <c r="Y14" s="75"/>
-      <c r="Z14" s="112"/>
+      <c r="Z14" s="99"/>
       <c r="AA14" s="14">
         <v>46060</v>
       </c>
@@ -2178,7 +2178,7 @@
       <c r="AC14" s="14"/>
       <c r="AD14" s="15"/>
       <c r="AE14" s="15"/>
-      <c r="AF14" s="111"/>
+      <c r="AF14" s="101"/>
       <c r="AG14" s="21">
         <v>46088</v>
       </c>
@@ -2186,7 +2186,7 @@
       <c r="AI14" s="14"/>
       <c r="AJ14" s="15"/>
       <c r="AK14" s="15"/>
-      <c r="AL14" s="111"/>
+      <c r="AL14" s="101"/>
       <c r="AM14" s="12">
         <v>46119</v>
       </c>
@@ -2208,7 +2208,7 @@
       <c r="E15" s="31"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="111"/>
+      <c r="H15" s="101"/>
       <c r="I15" s="12">
         <v>46030</v>
       </c>
@@ -2220,7 +2220,7 @@
         <v>7</v>
       </c>
       <c r="M15" s="2"/>
-      <c r="N15" s="111"/>
+      <c r="N15" s="101"/>
       <c r="O15" s="14">
         <v>46061</v>
       </c>
@@ -2228,13 +2228,13 @@
       <c r="Q15" s="18"/>
       <c r="R15" s="18"/>
       <c r="S15" s="18"/>
-      <c r="T15" s="115"/>
+      <c r="T15" s="96"/>
       <c r="U15" s="71"/>
       <c r="V15" s="76"/>
       <c r="W15" s="71"/>
       <c r="X15" s="75"/>
       <c r="Y15" s="75"/>
-      <c r="Z15" s="112"/>
+      <c r="Z15" s="99"/>
       <c r="AA15" s="14">
         <v>46061</v>
       </c>
@@ -2242,7 +2242,7 @@
       <c r="AC15" s="18"/>
       <c r="AD15" s="18"/>
       <c r="AE15" s="18"/>
-      <c r="AF15" s="111"/>
+      <c r="AF15" s="101"/>
       <c r="AG15" s="21">
         <v>46089</v>
       </c>
@@ -2250,7 +2250,7 @@
       <c r="AI15" s="18"/>
       <c r="AJ15" s="18"/>
       <c r="AK15" s="18"/>
-      <c r="AL15" s="111"/>
+      <c r="AL15" s="101"/>
       <c r="AM15" s="12">
         <v>46120</v>
       </c>
@@ -2272,7 +2272,7 @@
       <c r="E16" s="29"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="111"/>
+      <c r="H16" s="101"/>
       <c r="I16" s="12">
         <v>46031</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>7</v>
       </c>
       <c r="M16" s="2"/>
-      <c r="N16" s="111" t="s">
+      <c r="N16" s="101" t="s">
         <v>26</v>
       </c>
       <c r="O16" s="1">
@@ -2300,13 +2300,13 @@
         <v>7</v>
       </c>
       <c r="S16" s="2"/>
-      <c r="T16" s="115"/>
+      <c r="T16" s="96"/>
       <c r="U16" s="71"/>
       <c r="V16" s="76"/>
       <c r="W16" s="71"/>
       <c r="X16" s="75"/>
       <c r="Y16" s="75"/>
-      <c r="Z16" s="112" t="s">
+      <c r="Z16" s="99" t="s">
         <v>26</v>
       </c>
       <c r="AA16" s="1">
@@ -2320,7 +2320,7 @@
         <v>7</v>
       </c>
       <c r="AE16" s="2"/>
-      <c r="AF16" s="111" t="s">
+      <c r="AF16" s="101" t="s">
         <v>27</v>
       </c>
       <c r="AG16" s="12">
@@ -2334,7 +2334,7 @@
         <v>7</v>
       </c>
       <c r="AK16" s="2"/>
-      <c r="AL16" s="111"/>
+      <c r="AL16" s="101"/>
       <c r="AM16" s="12">
         <v>46121</v>
       </c>
@@ -2352,7 +2352,7 @@
       <c r="E17" s="29"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
-      <c r="H17" s="111"/>
+      <c r="H17" s="101"/>
       <c r="I17" s="21">
         <v>46032</v>
       </c>
@@ -2360,7 +2360,7 @@
       <c r="K17" s="14"/>
       <c r="L17" s="15"/>
       <c r="M17" s="20"/>
-      <c r="N17" s="111"/>
+      <c r="N17" s="101"/>
       <c r="O17" s="1">
         <v>46063</v>
       </c>
@@ -2374,13 +2374,13 @@
         <v>7</v>
       </c>
       <c r="S17" s="2"/>
-      <c r="T17" s="115"/>
+      <c r="T17" s="96"/>
       <c r="U17" s="71"/>
       <c r="V17" s="71"/>
       <c r="W17" s="71"/>
       <c r="X17" s="75"/>
       <c r="Y17" s="75"/>
-      <c r="Z17" s="112"/>
+      <c r="Z17" s="99"/>
       <c r="AA17" s="1">
         <v>46063</v>
       </c>
@@ -2392,7 +2392,7 @@
         <v>7</v>
       </c>
       <c r="AE17" s="2"/>
-      <c r="AF17" s="111"/>
+      <c r="AF17" s="101"/>
       <c r="AG17" s="12">
         <v>46091</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>7</v>
       </c>
       <c r="AK17" s="2"/>
-      <c r="AL17" s="111"/>
+      <c r="AL17" s="101"/>
       <c r="AM17" s="12">
         <v>46122</v>
       </c>
@@ -2424,7 +2424,7 @@
       <c r="E18" s="28"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="111"/>
+      <c r="H18" s="101"/>
       <c r="I18" s="21">
         <v>46033</v>
       </c>
@@ -2432,7 +2432,7 @@
       <c r="K18" s="16"/>
       <c r="L18" s="16"/>
       <c r="M18" s="36"/>
-      <c r="N18" s="111"/>
+      <c r="N18" s="101"/>
       <c r="O18" s="1">
         <v>46064</v>
       </c>
@@ -2446,13 +2446,13 @@
         <v>7</v>
       </c>
       <c r="S18" s="2"/>
-      <c r="T18" s="115"/>
+      <c r="T18" s="96"/>
       <c r="U18" s="71"/>
       <c r="V18" s="73"/>
       <c r="W18" s="73"/>
       <c r="X18" s="73"/>
       <c r="Y18" s="73"/>
-      <c r="Z18" s="112"/>
+      <c r="Z18" s="99"/>
       <c r="AA18" s="1">
         <v>46064</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>7</v>
       </c>
       <c r="AE18" s="2"/>
-      <c r="AF18" s="111"/>
+      <c r="AF18" s="101"/>
       <c r="AG18" s="12">
         <v>46092</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>7</v>
       </c>
       <c r="AK18" s="2"/>
-      <c r="AL18" s="111"/>
+      <c r="AL18" s="101"/>
       <c r="AM18" s="21">
         <v>46123</v>
       </c>
@@ -2494,7 +2494,7 @@
       <c r="E19" s="29"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
-      <c r="H19" s="111" t="s">
+      <c r="H19" s="101" t="s">
         <v>29</v>
       </c>
       <c r="I19" s="12">
@@ -2508,7 +2508,7 @@
         <v>7</v>
       </c>
       <c r="M19" s="35"/>
-      <c r="N19" s="111"/>
+      <c r="N19" s="101"/>
       <c r="O19" s="1">
         <v>46065</v>
       </c>
@@ -2522,13 +2522,13 @@
         <v>7</v>
       </c>
       <c r="S19" s="2"/>
-      <c r="T19" s="115"/>
+      <c r="T19" s="96"/>
       <c r="U19" s="71"/>
       <c r="V19" s="76"/>
       <c r="W19" s="71"/>
       <c r="X19" s="75"/>
       <c r="Y19" s="75"/>
-      <c r="Z19" s="112"/>
+      <c r="Z19" s="99"/>
       <c r="AA19" s="1">
         <v>46065</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>7</v>
       </c>
       <c r="AE19" s="2"/>
-      <c r="AF19" s="111"/>
+      <c r="AF19" s="101"/>
       <c r="AG19" s="12">
         <v>46093</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>7</v>
       </c>
       <c r="AK19" s="2"/>
-      <c r="AL19" s="111"/>
+      <c r="AL19" s="101"/>
       <c r="AM19" s="21">
         <v>46124</v>
       </c>
@@ -2570,7 +2570,7 @@
       <c r="E20" s="17"/>
       <c r="F20" s="15"/>
       <c r="G20" s="15"/>
-      <c r="H20" s="111"/>
+      <c r="H20" s="101"/>
       <c r="I20" s="12">
         <v>46035</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>7</v>
       </c>
       <c r="M20" s="35"/>
-      <c r="N20" s="111"/>
+      <c r="N20" s="101"/>
       <c r="O20" s="1">
         <v>46066</v>
       </c>
@@ -2594,13 +2594,13 @@
         <v>7</v>
       </c>
       <c r="S20" s="2"/>
-      <c r="T20" s="115"/>
+      <c r="T20" s="96"/>
       <c r="U20" s="71"/>
       <c r="V20" s="76"/>
       <c r="W20" s="76"/>
       <c r="X20" s="75"/>
       <c r="Y20" s="75"/>
-      <c r="Z20" s="112"/>
+      <c r="Z20" s="99"/>
       <c r="AA20" s="1">
         <v>46066</v>
       </c>
@@ -2612,7 +2612,7 @@
         <v>7</v>
       </c>
       <c r="AE20" s="2"/>
-      <c r="AF20" s="111"/>
+      <c r="AF20" s="101"/>
       <c r="AG20" s="12">
         <v>46094</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>7</v>
       </c>
       <c r="AK20" s="2"/>
-      <c r="AL20" s="111" t="s">
+      <c r="AL20" s="101" t="s">
         <v>30</v>
       </c>
       <c r="AM20" s="12">
@@ -2644,7 +2644,7 @@
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
-      <c r="H21" s="111"/>
+      <c r="H21" s="101"/>
       <c r="I21" s="12">
         <v>46036</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>7</v>
       </c>
       <c r="M21" s="35"/>
-      <c r="N21" s="111"/>
+      <c r="N21" s="101"/>
       <c r="O21" s="14">
         <v>46067</v>
       </c>
@@ -2664,13 +2664,13 @@
       <c r="Q21" s="14"/>
       <c r="R21" s="15"/>
       <c r="S21" s="15"/>
-      <c r="T21" s="115"/>
+      <c r="T21" s="96"/>
       <c r="U21" s="71"/>
       <c r="V21" s="76"/>
       <c r="W21" s="76"/>
       <c r="X21" s="75"/>
       <c r="Y21" s="75"/>
-      <c r="Z21" s="112"/>
+      <c r="Z21" s="99"/>
       <c r="AA21" s="14">
         <v>46067</v>
       </c>
@@ -2678,7 +2678,7 @@
       <c r="AC21" s="14"/>
       <c r="AD21" s="15"/>
       <c r="AE21" s="15"/>
-      <c r="AF21" s="111"/>
+      <c r="AF21" s="101"/>
       <c r="AG21" s="21">
         <v>46095</v>
       </c>
@@ -2686,7 +2686,7 @@
       <c r="AI21" s="14"/>
       <c r="AJ21" s="15"/>
       <c r="AK21" s="15"/>
-      <c r="AL21" s="111"/>
+      <c r="AL21" s="101"/>
       <c r="AM21" s="12">
         <v>46126</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>7</v>
       </c>
       <c r="G22" s="2"/>
-      <c r="H22" s="111"/>
+      <c r="H22" s="101"/>
       <c r="I22" s="12">
         <v>46037</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>7</v>
       </c>
       <c r="M22" s="35"/>
-      <c r="N22" s="111"/>
+      <c r="N22" s="101"/>
       <c r="O22" s="14">
         <v>46068</v>
       </c>
@@ -2730,13 +2730,13 @@
       <c r="Q22" s="14"/>
       <c r="R22" s="15"/>
       <c r="S22" s="15"/>
-      <c r="T22" s="115"/>
+      <c r="T22" s="96"/>
       <c r="U22" s="71"/>
       <c r="V22" s="76"/>
       <c r="W22" s="76"/>
       <c r="X22" s="75"/>
       <c r="Y22" s="75"/>
-      <c r="Z22" s="112"/>
+      <c r="Z22" s="99"/>
       <c r="AA22" s="14">
         <v>46068</v>
       </c>
@@ -2744,7 +2744,7 @@
       <c r="AC22" s="14"/>
       <c r="AD22" s="15"/>
       <c r="AE22" s="15"/>
-      <c r="AF22" s="111"/>
+      <c r="AF22" s="101"/>
       <c r="AG22" s="21">
         <v>46096</v>
       </c>
@@ -2752,7 +2752,7 @@
       <c r="AI22" s="14"/>
       <c r="AJ22" s="15"/>
       <c r="AK22" s="15"/>
-      <c r="AL22" s="111"/>
+      <c r="AL22" s="101"/>
       <c r="AM22" s="12">
         <v>46127</v>
       </c>
@@ -2776,7 +2776,7 @@
         <v>7</v>
       </c>
       <c r="G23" s="2"/>
-      <c r="H23" s="111"/>
+      <c r="H23" s="101"/>
       <c r="I23" s="12">
         <v>46038</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>7</v>
       </c>
       <c r="M23" s="35"/>
-      <c r="N23" s="111" t="s">
+      <c r="N23" s="101" t="s">
         <v>32</v>
       </c>
       <c r="O23" s="1">
@@ -2800,13 +2800,13 @@
       <c r="Q23" s="3"/>
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
-      <c r="T23" s="115"/>
+      <c r="T23" s="96"/>
       <c r="U23" s="71"/>
       <c r="V23" s="76"/>
       <c r="W23" s="71"/>
       <c r="X23" s="75"/>
       <c r="Y23" s="75"/>
-      <c r="Z23" s="112" t="s">
+      <c r="Z23" s="99" t="s">
         <v>32</v>
       </c>
       <c r="AA23" s="1">
@@ -2820,7 +2820,7 @@
       <c r="AE23" s="2">
         <v>7</v>
       </c>
-      <c r="AF23" s="111" t="s">
+      <c r="AF23" s="101" t="s">
         <v>33</v>
       </c>
       <c r="AG23" s="12">
@@ -2834,7 +2834,7 @@
         <v>7</v>
       </c>
       <c r="AK23" s="2"/>
-      <c r="AL23" s="111"/>
+      <c r="AL23" s="101"/>
       <c r="AM23" s="12">
         <v>46128</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>7</v>
       </c>
       <c r="G24" s="2"/>
-      <c r="H24" s="111"/>
+      <c r="H24" s="101"/>
       <c r="I24" s="21">
         <v>46039</v>
       </c>
@@ -2866,7 +2866,7 @@
       <c r="K24" s="14"/>
       <c r="L24" s="15"/>
       <c r="M24" s="20"/>
-      <c r="N24" s="111"/>
+      <c r="N24" s="101"/>
       <c r="O24" s="1">
         <v>46070</v>
       </c>
@@ -2874,13 +2874,13 @@
       <c r="Q24" s="3"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
-      <c r="T24" s="115"/>
+      <c r="T24" s="96"/>
       <c r="U24" s="71"/>
       <c r="V24" s="71"/>
       <c r="W24" s="71"/>
       <c r="X24" s="75"/>
       <c r="Y24" s="75"/>
-      <c r="Z24" s="112"/>
+      <c r="Z24" s="99"/>
       <c r="AA24" s="1">
         <v>46070</v>
       </c>
@@ -2892,7 +2892,7 @@
       <c r="AE24" s="2">
         <v>7</v>
       </c>
-      <c r="AF24" s="111"/>
+      <c r="AF24" s="101"/>
       <c r="AG24" s="12">
         <v>46098</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>7</v>
       </c>
       <c r="AK24" s="2"/>
-      <c r="AL24" s="111"/>
+      <c r="AL24" s="101"/>
       <c r="AM24" s="12">
         <v>46129</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>7</v>
       </c>
       <c r="G25" s="2"/>
-      <c r="H25" s="111"/>
+      <c r="H25" s="101"/>
       <c r="I25" s="21">
         <v>46040</v>
       </c>
@@ -2938,7 +2938,7 @@
       <c r="K25" s="17"/>
       <c r="L25" s="15"/>
       <c r="M25" s="26"/>
-      <c r="N25" s="111"/>
+      <c r="N25" s="101"/>
       <c r="O25" s="1">
         <v>46071</v>
       </c>
@@ -2946,13 +2946,13 @@
       <c r="Q25" s="3"/>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
-      <c r="T25" s="115"/>
+      <c r="T25" s="96"/>
       <c r="U25" s="71"/>
       <c r="V25" s="76"/>
       <c r="W25" s="76"/>
       <c r="X25" s="75"/>
       <c r="Y25" s="72"/>
-      <c r="Z25" s="112"/>
+      <c r="Z25" s="99"/>
       <c r="AA25" s="1">
         <v>46071</v>
       </c>
@@ -2964,7 +2964,7 @@
       <c r="AE25" s="2">
         <v>7</v>
       </c>
-      <c r="AF25" s="111"/>
+      <c r="AF25" s="101"/>
       <c r="AG25" s="12">
         <v>46099</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>7</v>
       </c>
       <c r="AK25" s="2"/>
-      <c r="AL25" s="111"/>
+      <c r="AL25" s="101"/>
       <c r="AM25" s="21">
         <v>46130</v>
       </c>
@@ -3000,7 +3000,7 @@
         <v>7</v>
       </c>
       <c r="G26" s="2"/>
-      <c r="H26" s="111" t="s">
+      <c r="H26" s="101" t="s">
         <v>34</v>
       </c>
       <c r="I26" s="12">
@@ -3014,7 +3014,7 @@
         <v>7</v>
       </c>
       <c r="M26" s="35"/>
-      <c r="N26" s="111"/>
+      <c r="N26" s="101"/>
       <c r="O26" s="1">
         <v>46072</v>
       </c>
@@ -3022,13 +3022,13 @@
       <c r="Q26" s="3"/>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
-      <c r="T26" s="115"/>
+      <c r="T26" s="96"/>
       <c r="U26" s="71"/>
       <c r="V26" s="77"/>
       <c r="W26" s="76"/>
       <c r="X26" s="75"/>
       <c r="Y26" s="75"/>
-      <c r="Z26" s="112"/>
+      <c r="Z26" s="99"/>
       <c r="AA26" s="1">
         <v>46072</v>
       </c>
@@ -3040,7 +3040,7 @@
       <c r="AE26" s="2">
         <v>7</v>
       </c>
-      <c r="AF26" s="111"/>
+      <c r="AF26" s="101"/>
       <c r="AG26" s="12">
         <v>46100</v>
       </c>
@@ -3052,7 +3052,7 @@
         <v>7</v>
       </c>
       <c r="AK26" s="2"/>
-      <c r="AL26" s="111"/>
+      <c r="AL26" s="101"/>
       <c r="AM26" s="21">
         <v>46131</v>
       </c>
@@ -3070,7 +3070,7 @@
       <c r="E27" s="17"/>
       <c r="F27" s="15"/>
       <c r="G27" s="15"/>
-      <c r="H27" s="111"/>
+      <c r="H27" s="101"/>
       <c r="I27" s="12">
         <v>46042</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>7</v>
       </c>
       <c r="M27" s="35"/>
-      <c r="N27" s="111"/>
+      <c r="N27" s="101"/>
       <c r="O27" s="1">
         <v>46073</v>
       </c>
@@ -3090,13 +3090,13 @@
       <c r="Q27" s="3"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
-      <c r="T27" s="115"/>
+      <c r="T27" s="96"/>
       <c r="U27" s="71"/>
       <c r="V27" s="77"/>
       <c r="W27" s="76"/>
       <c r="X27" s="75"/>
       <c r="Y27" s="75"/>
-      <c r="Z27" s="112"/>
+      <c r="Z27" s="99"/>
       <c r="AA27" s="1">
         <v>46073</v>
       </c>
@@ -3108,7 +3108,7 @@
       <c r="AE27" s="2">
         <v>7</v>
       </c>
-      <c r="AF27" s="111"/>
+      <c r="AF27" s="101"/>
       <c r="AG27" s="12">
         <v>46101</v>
       </c>
@@ -3120,7 +3120,7 @@
         <v>7</v>
       </c>
       <c r="AK27" s="2"/>
-      <c r="AL27" s="111" t="s">
+      <c r="AL27" s="101" t="s">
         <v>35</v>
       </c>
       <c r="AM27" s="12">
@@ -3140,7 +3140,7 @@
       <c r="E28" s="14"/>
       <c r="F28" s="15"/>
       <c r="G28" s="15"/>
-      <c r="H28" s="111"/>
+      <c r="H28" s="101"/>
       <c r="I28" s="12">
         <v>46043</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>7</v>
       </c>
       <c r="M28" s="35"/>
-      <c r="N28" s="111"/>
+      <c r="N28" s="101"/>
       <c r="O28" s="14">
         <v>46074</v>
       </c>
@@ -3160,13 +3160,13 @@
       <c r="Q28" s="14"/>
       <c r="R28" s="15"/>
       <c r="S28" s="15"/>
-      <c r="T28" s="115"/>
+      <c r="T28" s="96"/>
       <c r="U28" s="71"/>
       <c r="V28" s="76"/>
       <c r="W28" s="76"/>
       <c r="X28" s="75"/>
       <c r="Y28" s="75"/>
-      <c r="Z28" s="112"/>
+      <c r="Z28" s="99"/>
       <c r="AA28" s="14">
         <v>46074</v>
       </c>
@@ -3174,7 +3174,7 @@
       <c r="AC28" s="14"/>
       <c r="AD28" s="15"/>
       <c r="AE28" s="15"/>
-      <c r="AF28" s="111"/>
+      <c r="AF28" s="101"/>
       <c r="AG28" s="21">
         <v>46102</v>
       </c>
@@ -3182,7 +3182,7 @@
       <c r="AI28" s="14"/>
       <c r="AJ28" s="15"/>
       <c r="AK28" s="15"/>
-      <c r="AL28" s="111"/>
+      <c r="AL28" s="101"/>
       <c r="AM28" s="12">
         <v>46133</v>
       </c>
@@ -3202,7 +3202,7 @@
       <c r="E29" s="49"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15"/>
-      <c r="H29" s="111"/>
+      <c r="H29" s="101"/>
       <c r="I29" s="12">
         <v>46044</v>
       </c>
@@ -3214,7 +3214,7 @@
         <v>7</v>
       </c>
       <c r="M29" s="35"/>
-      <c r="N29" s="111"/>
+      <c r="N29" s="101"/>
       <c r="O29" s="14">
         <v>46075</v>
       </c>
@@ -3222,13 +3222,13 @@
       <c r="Q29" s="14"/>
       <c r="R29" s="15"/>
       <c r="S29" s="15"/>
-      <c r="T29" s="115"/>
+      <c r="T29" s="96"/>
       <c r="U29" s="71"/>
       <c r="V29" s="76"/>
       <c r="W29" s="76"/>
       <c r="X29" s="75"/>
       <c r="Y29" s="75"/>
-      <c r="Z29" s="112"/>
+      <c r="Z29" s="99"/>
       <c r="AA29" s="14">
         <v>46075</v>
       </c>
@@ -3236,7 +3236,7 @@
       <c r="AC29" s="14"/>
       <c r="AD29" s="15"/>
       <c r="AE29" s="15"/>
-      <c r="AF29" s="111"/>
+      <c r="AF29" s="101"/>
       <c r="AG29" s="21">
         <v>46103</v>
       </c>
@@ -3244,7 +3244,7 @@
       <c r="AI29" s="14"/>
       <c r="AJ29" s="15"/>
       <c r="AK29" s="15"/>
-      <c r="AL29" s="111"/>
+      <c r="AL29" s="101"/>
       <c r="AM29" s="12">
         <v>46134</v>
       </c>
@@ -3262,7 +3262,7 @@
       <c r="E30" s="51"/>
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
-      <c r="H30" s="111"/>
+      <c r="H30" s="101"/>
       <c r="I30" s="12">
         <v>46045</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>7</v>
       </c>
       <c r="M30" s="35"/>
-      <c r="N30" s="111" t="s">
+      <c r="N30" s="101" t="s">
         <v>38</v>
       </c>
       <c r="O30" s="1">
@@ -3284,13 +3284,13 @@
       <c r="Q30" s="1"/>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
-      <c r="T30" s="115"/>
+      <c r="T30" s="96"/>
       <c r="U30" s="71"/>
       <c r="V30" s="76"/>
       <c r="W30" s="76"/>
       <c r="X30" s="75"/>
       <c r="Y30" s="75"/>
-      <c r="Z30" s="112" t="s">
+      <c r="Z30" s="99" t="s">
         <v>38</v>
       </c>
       <c r="AA30" s="1">
@@ -3304,7 +3304,7 @@
       <c r="AE30" s="2">
         <v>7</v>
       </c>
-      <c r="AF30" s="111" t="s">
+      <c r="AF30" s="101" t="s">
         <v>39</v>
       </c>
       <c r="AG30" s="12">
@@ -3318,7 +3318,7 @@
         <v>7</v>
       </c>
       <c r="AK30" s="2"/>
-      <c r="AL30" s="111"/>
+      <c r="AL30" s="101"/>
       <c r="AM30" s="12">
         <v>46135</v>
       </c>
@@ -3336,7 +3336,7 @@
       <c r="E31" s="51"/>
       <c r="F31" s="15"/>
       <c r="G31" s="15"/>
-      <c r="H31" s="111"/>
+      <c r="H31" s="101"/>
       <c r="I31" s="21">
         <v>46046</v>
       </c>
@@ -3344,7 +3344,7 @@
       <c r="K31" s="14"/>
       <c r="L31" s="15"/>
       <c r="M31" s="20"/>
-      <c r="N31" s="111"/>
+      <c r="N31" s="101"/>
       <c r="O31" s="1">
         <v>46077</v>
       </c>
@@ -3352,13 +3352,13 @@
       <c r="Q31" s="1"/>
       <c r="R31" s="2"/>
       <c r="S31" s="2"/>
-      <c r="T31" s="115"/>
+      <c r="T31" s="96"/>
       <c r="U31" s="71"/>
       <c r="V31" s="71"/>
       <c r="W31" s="71"/>
       <c r="X31" s="75"/>
       <c r="Y31" s="75"/>
-      <c r="Z31" s="112"/>
+      <c r="Z31" s="99"/>
       <c r="AA31" s="1">
         <v>46077</v>
       </c>
@@ -3370,7 +3370,7 @@
       <c r="AE31" s="2">
         <v>7</v>
       </c>
-      <c r="AF31" s="111"/>
+      <c r="AF31" s="101"/>
       <c r="AG31" s="12">
         <v>46105</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>7</v>
       </c>
       <c r="AK31" s="2"/>
-      <c r="AL31" s="111"/>
+      <c r="AL31" s="101"/>
       <c r="AM31" s="12">
         <v>46136</v>
       </c>
@@ -3402,7 +3402,7 @@
       <c r="E32" s="51"/>
       <c r="F32" s="15"/>
       <c r="G32" s="15"/>
-      <c r="H32" s="111"/>
+      <c r="H32" s="101"/>
       <c r="I32" s="21">
         <v>46047</v>
       </c>
@@ -3410,7 +3410,7 @@
       <c r="K32" s="17"/>
       <c r="L32" s="15"/>
       <c r="M32" s="20"/>
-      <c r="N32" s="111"/>
+      <c r="N32" s="101"/>
       <c r="O32" s="1">
         <v>46078</v>
       </c>
@@ -3418,13 +3418,13 @@
       <c r="Q32" s="1"/>
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
-      <c r="T32" s="115"/>
+      <c r="T32" s="96"/>
       <c r="U32" s="71"/>
       <c r="V32" s="76"/>
       <c r="W32" s="76"/>
       <c r="X32" s="75"/>
       <c r="Y32" s="75"/>
-      <c r="Z32" s="112"/>
+      <c r="Z32" s="99"/>
       <c r="AA32" s="1">
         <v>46078</v>
       </c>
@@ -3436,7 +3436,7 @@
       <c r="AE32" s="2">
         <v>7</v>
       </c>
-      <c r="AF32" s="111"/>
+      <c r="AF32" s="101"/>
       <c r="AG32" s="12">
         <v>46106</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>7</v>
       </c>
       <c r="AK32" s="2"/>
-      <c r="AL32" s="111"/>
+      <c r="AL32" s="101"/>
       <c r="AM32" s="21">
         <v>46137</v>
       </c>
@@ -3466,7 +3466,7 @@
       <c r="E33" s="53"/>
       <c r="F33" s="18"/>
       <c r="G33" s="18"/>
-      <c r="H33" s="108" t="s">
+      <c r="H33" s="105" t="s">
         <v>40</v>
       </c>
       <c r="I33" s="12">
@@ -3482,7 +3482,7 @@
         <v>7</v>
       </c>
       <c r="M33" s="2"/>
-      <c r="N33" s="111"/>
+      <c r="N33" s="101"/>
       <c r="O33" s="1">
         <v>46079</v>
       </c>
@@ -3490,13 +3490,13 @@
       <c r="Q33" s="4"/>
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
-      <c r="T33" s="115"/>
+      <c r="T33" s="96"/>
       <c r="U33" s="71"/>
       <c r="V33" s="76"/>
       <c r="W33" s="76"/>
       <c r="X33" s="75"/>
       <c r="Y33" s="75"/>
-      <c r="Z33" s="112"/>
+      <c r="Z33" s="99"/>
       <c r="AA33" s="1">
         <v>46079</v>
       </c>
@@ -3508,7 +3508,7 @@
       <c r="AE33" s="2">
         <v>7</v>
       </c>
-      <c r="AF33" s="111"/>
+      <c r="AF33" s="101"/>
       <c r="AG33" s="12">
         <v>46107</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>7</v>
       </c>
       <c r="AK33" s="4"/>
-      <c r="AL33" s="111"/>
+      <c r="AL33" s="101"/>
       <c r="AM33" s="21">
         <v>46138</v>
       </c>
@@ -3540,7 +3540,7 @@
       <c r="E34" s="14"/>
       <c r="F34" s="15"/>
       <c r="G34" s="15"/>
-      <c r="H34" s="119"/>
+      <c r="H34" s="106"/>
       <c r="I34" s="12">
         <v>46049</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>7</v>
       </c>
       <c r="M34" s="2"/>
-      <c r="N34" s="111"/>
+      <c r="N34" s="101"/>
       <c r="O34" s="1">
         <v>46080</v>
       </c>
@@ -3562,13 +3562,13 @@
       <c r="Q34" s="1"/>
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
-      <c r="T34" s="115"/>
+      <c r="T34" s="96"/>
       <c r="U34" s="71"/>
       <c r="V34" s="76"/>
       <c r="W34" s="76"/>
       <c r="X34" s="75"/>
       <c r="Y34" s="75"/>
-      <c r="Z34" s="112"/>
+      <c r="Z34" s="99"/>
       <c r="AA34" s="1">
         <v>46080</v>
       </c>
@@ -3580,7 +3580,7 @@
       <c r="AE34" s="2">
         <v>7</v>
       </c>
-      <c r="AF34" s="111"/>
+      <c r="AF34" s="101"/>
       <c r="AG34" s="12">
         <v>46108</v>
       </c>
@@ -3594,7 +3594,7 @@
         <v>7</v>
       </c>
       <c r="AK34" s="2"/>
-      <c r="AL34" s="111" t="s">
+      <c r="AL34" s="101" t="s">
         <v>41</v>
       </c>
       <c r="AM34" s="12">
@@ -3614,7 +3614,7 @@
       <c r="E35" s="14"/>
       <c r="F35" s="15"/>
       <c r="G35" s="15"/>
-      <c r="H35" s="119"/>
+      <c r="H35" s="106"/>
       <c r="I35" s="12">
         <v>46050</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>7</v>
       </c>
       <c r="M35" s="2"/>
-      <c r="N35" s="111"/>
+      <c r="N35" s="101"/>
       <c r="O35" s="14">
         <v>46081</v>
       </c>
@@ -3636,13 +3636,13 @@
       <c r="Q35" s="14"/>
       <c r="R35" s="15"/>
       <c r="S35" s="15"/>
-      <c r="T35" s="115"/>
+      <c r="T35" s="96"/>
       <c r="U35" s="71"/>
       <c r="V35" s="76"/>
       <c r="W35" s="76"/>
       <c r="X35" s="75"/>
       <c r="Y35" s="75"/>
-      <c r="Z35" s="112"/>
+      <c r="Z35" s="99"/>
       <c r="AA35" s="14">
         <v>46081</v>
       </c>
@@ -3650,7 +3650,7 @@
       <c r="AC35" s="14"/>
       <c r="AD35" s="15"/>
       <c r="AE35" s="15"/>
-      <c r="AF35" s="111"/>
+      <c r="AF35" s="101"/>
       <c r="AG35" s="21">
         <v>46109</v>
       </c>
@@ -3658,7 +3658,7 @@
       <c r="AI35" s="14"/>
       <c r="AJ35" s="15"/>
       <c r="AK35" s="15"/>
-      <c r="AL35" s="111"/>
+      <c r="AL35" s="101"/>
       <c r="AM35" s="12">
         <v>46140</v>
       </c>
@@ -3678,7 +3678,7 @@
       <c r="E36" s="55"/>
       <c r="F36" s="19"/>
       <c r="G36" s="19"/>
-      <c r="H36" s="119"/>
+      <c r="H36" s="106"/>
       <c r="I36" s="12">
         <v>46051</v>
       </c>
@@ -3692,25 +3692,25 @@
         <v>7</v>
       </c>
       <c r="M36" s="2"/>
-      <c r="N36" s="111"/>
-      <c r="O36" s="111"/>
-      <c r="P36" s="111"/>
-      <c r="Q36" s="111"/>
-      <c r="R36" s="111"/>
-      <c r="S36" s="111"/>
-      <c r="T36" s="115"/>
+      <c r="N36" s="101"/>
+      <c r="O36" s="101"/>
+      <c r="P36" s="101"/>
+      <c r="Q36" s="101"/>
+      <c r="R36" s="101"/>
+      <c r="S36" s="101"/>
+      <c r="T36" s="96"/>
       <c r="U36" s="71"/>
       <c r="V36" s="3"/>
       <c r="W36" s="76"/>
       <c r="X36" s="75"/>
       <c r="Y36" s="75"/>
-      <c r="Z36" s="112"/>
-      <c r="AA36" s="111"/>
-      <c r="AB36" s="111"/>
-      <c r="AC36" s="111"/>
-      <c r="AD36" s="111"/>
-      <c r="AE36" s="111"/>
-      <c r="AF36" s="111"/>
+      <c r="Z36" s="99"/>
+      <c r="AA36" s="101"/>
+      <c r="AB36" s="101"/>
+      <c r="AC36" s="101"/>
+      <c r="AD36" s="101"/>
+      <c r="AE36" s="101"/>
+      <c r="AF36" s="101"/>
       <c r="AG36" s="21">
         <v>46110</v>
       </c>
@@ -3718,7 +3718,7 @@
       <c r="AI36" s="19"/>
       <c r="AJ36" s="19"/>
       <c r="AK36" s="19"/>
-      <c r="AL36" s="111"/>
+      <c r="AL36" s="101"/>
       <c r="AM36" s="12">
         <v>46141</v>
       </c>
@@ -3736,7 +3736,7 @@
       <c r="E37" s="57"/>
       <c r="F37" s="19"/>
       <c r="G37" s="19"/>
-      <c r="H37" s="119"/>
+      <c r="H37" s="106"/>
       <c r="I37" s="12">
         <v>46052</v>
       </c>
@@ -3750,25 +3750,25 @@
         <v>7</v>
       </c>
       <c r="M37" s="2"/>
-      <c r="N37" s="111"/>
-      <c r="O37" s="111"/>
-      <c r="P37" s="111"/>
-      <c r="Q37" s="111"/>
-      <c r="R37" s="111"/>
-      <c r="S37" s="111"/>
-      <c r="T37" s="115"/>
+      <c r="N37" s="101"/>
+      <c r="O37" s="101"/>
+      <c r="P37" s="101"/>
+      <c r="Q37" s="101"/>
+      <c r="R37" s="101"/>
+      <c r="S37" s="101"/>
+      <c r="T37" s="96"/>
       <c r="U37" s="71"/>
       <c r="V37" s="76"/>
       <c r="W37" s="71"/>
       <c r="X37" s="75"/>
       <c r="Y37" s="75"/>
-      <c r="Z37" s="112"/>
-      <c r="AA37" s="111"/>
-      <c r="AB37" s="111"/>
-      <c r="AC37" s="111"/>
-      <c r="AD37" s="111"/>
-      <c r="AE37" s="111"/>
-      <c r="AF37" s="108"/>
+      <c r="Z37" s="99"/>
+      <c r="AA37" s="101"/>
+      <c r="AB37" s="101"/>
+      <c r="AC37" s="101"/>
+      <c r="AD37" s="101"/>
+      <c r="AE37" s="101"/>
+      <c r="AF37" s="105"/>
       <c r="AG37" s="12">
         <v>46111</v>
       </c>
@@ -3780,7 +3780,7 @@
         <v>7</v>
       </c>
       <c r="AK37" s="8"/>
-      <c r="AL37" s="111"/>
+      <c r="AL37" s="101"/>
       <c r="AM37" s="12">
         <v>46142</v>
       </c>
@@ -3798,7 +3798,7 @@
       <c r="E38" s="59"/>
       <c r="F38" s="19"/>
       <c r="G38" s="19"/>
-      <c r="H38" s="109"/>
+      <c r="H38" s="107"/>
       <c r="I38" s="21">
         <v>46053</v>
       </c>
@@ -3806,25 +3806,25 @@
       <c r="K38" s="37"/>
       <c r="L38" s="38"/>
       <c r="M38" s="38"/>
-      <c r="N38" s="111"/>
-      <c r="O38" s="111"/>
-      <c r="P38" s="111"/>
-      <c r="Q38" s="111"/>
-      <c r="R38" s="111"/>
-      <c r="S38" s="111"/>
-      <c r="T38" s="115"/>
+      <c r="N38" s="101"/>
+      <c r="O38" s="101"/>
+      <c r="P38" s="101"/>
+      <c r="Q38" s="101"/>
+      <c r="R38" s="101"/>
+      <c r="S38" s="101"/>
+      <c r="T38" s="96"/>
       <c r="U38" s="71"/>
       <c r="V38" s="78"/>
       <c r="W38" s="78"/>
       <c r="X38" s="79"/>
       <c r="Y38" s="79"/>
-      <c r="Z38" s="112"/>
-      <c r="AA38" s="111"/>
-      <c r="AB38" s="111"/>
-      <c r="AC38" s="111"/>
-      <c r="AD38" s="111"/>
-      <c r="AE38" s="111"/>
-      <c r="AF38" s="109"/>
+      <c r="Z38" s="99"/>
+      <c r="AA38" s="101"/>
+      <c r="AB38" s="101"/>
+      <c r="AC38" s="101"/>
+      <c r="AD38" s="101"/>
+      <c r="AE38" s="101"/>
+      <c r="AF38" s="107"/>
       <c r="AG38" s="1">
         <v>46112</v>
       </c>
@@ -3836,12 +3836,12 @@
         <v>7</v>
       </c>
       <c r="AK38" s="8"/>
-      <c r="AL38" s="120"/>
-      <c r="AM38" s="121"/>
-      <c r="AN38" s="121"/>
-      <c r="AO38" s="121"/>
-      <c r="AP38" s="121"/>
-      <c r="AQ38" s="112"/>
+      <c r="AL38" s="97"/>
+      <c r="AM38" s="98"/>
+      <c r="AN38" s="98"/>
+      <c r="AO38" s="98"/>
+      <c r="AP38" s="98"/>
+      <c r="AQ38" s="99"/>
     </row>
     <row r="39" spans="2:43" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="11"/>
@@ -3984,103 +3984,86 @@
       <c r="D42" s="88" t="s">
         <v>58</v>
       </c>
-      <c r="J42" s="102" t="s">
+      <c r="J42" s="108" t="s">
         <v>47</v>
       </c>
-      <c r="K42" s="103"/>
-      <c r="P42" s="98" t="s">
+      <c r="K42" s="109"/>
+      <c r="P42" s="119" t="s">
         <v>72</v>
       </c>
-      <c r="Q42" s="99"/>
+      <c r="Q42" s="120"/>
     </row>
     <row r="43" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D43" s="90" t="s">
         <v>59</v>
       </c>
-      <c r="J43" s="104"/>
-      <c r="K43" s="105"/>
-      <c r="P43" s="100" t="s">
+      <c r="J43" s="110"/>
+      <c r="K43" s="111"/>
+      <c r="P43" s="121" t="s">
         <v>79</v>
       </c>
-      <c r="Q43" s="101"/>
+      <c r="Q43" s="122"/>
     </row>
     <row r="44" spans="2:43" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D44" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="J44" s="106"/>
-      <c r="K44" s="107"/>
-      <c r="P44" s="100" t="s">
+      <c r="J44" s="112"/>
+      <c r="K44" s="113"/>
+      <c r="P44" s="121" t="s">
         <v>73</v>
       </c>
-      <c r="Q44" s="101"/>
+      <c r="Q44" s="122"/>
     </row>
     <row r="45" spans="2:43" x14ac:dyDescent="0.25">
       <c r="D45" s="91" t="s">
         <v>61</v>
       </c>
-      <c r="P45" s="100" t="s">
+      <c r="P45" s="121" t="s">
         <v>74</v>
       </c>
-      <c r="Q45" s="101"/>
+      <c r="Q45" s="122"/>
     </row>
     <row r="46" spans="2:43" x14ac:dyDescent="0.25">
-      <c r="P46" s="100" t="s">
+      <c r="P46" s="121" t="s">
         <v>75</v>
       </c>
-      <c r="Q46" s="101"/>
+      <c r="Q46" s="122"/>
     </row>
     <row r="47" spans="2:43" x14ac:dyDescent="0.25">
       <c r="D47" s="95" t="s">
         <v>80</v>
       </c>
-      <c r="P47" s="100" t="s">
+      <c r="P47" s="121" t="s">
         <v>76</v>
       </c>
-      <c r="Q47" s="101"/>
+      <c r="Q47" s="122"/>
     </row>
     <row r="48" spans="2:43" x14ac:dyDescent="0.25">
       <c r="D48" s="95" t="s">
         <v>81</v>
       </c>
-      <c r="P48" s="96" t="s">
+      <c r="P48" s="117" t="s">
         <v>77</v>
       </c>
-      <c r="Q48" s="97"/>
+      <c r="Q48" s="118"/>
     </row>
     <row r="49" spans="16:17" x14ac:dyDescent="0.25">
-      <c r="P49" s="96" t="s">
+      <c r="P49" s="117" t="s">
         <v>78</v>
       </c>
-      <c r="Q49" s="97"/>
+      <c r="Q49" s="118"/>
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="T8:T11"/>
-    <mergeCell ref="AL38:AQ38"/>
-    <mergeCell ref="AL6:AQ6"/>
-    <mergeCell ref="AL8:AL12"/>
-    <mergeCell ref="AL13:AL19"/>
-    <mergeCell ref="AN13:AO13"/>
-    <mergeCell ref="AL20:AL26"/>
-    <mergeCell ref="AL27:AL33"/>
-    <mergeCell ref="AL34:AL37"/>
-    <mergeCell ref="T19:T25"/>
-    <mergeCell ref="Z23:Z29"/>
-    <mergeCell ref="T26:T32"/>
-    <mergeCell ref="Z30:Z35"/>
-    <mergeCell ref="Z16:Z22"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="N9:N15"/>
-    <mergeCell ref="H12:H18"/>
-    <mergeCell ref="N16:N22"/>
-    <mergeCell ref="H19:H25"/>
-    <mergeCell ref="N23:N29"/>
-    <mergeCell ref="H26:H32"/>
-    <mergeCell ref="N30:N35"/>
-    <mergeCell ref="H33:H38"/>
-    <mergeCell ref="N36:S38"/>
+    <mergeCell ref="P48:Q48"/>
+    <mergeCell ref="P49:Q49"/>
+    <mergeCell ref="P42:Q42"/>
+    <mergeCell ref="P44:Q44"/>
+    <mergeCell ref="P45:Q45"/>
+    <mergeCell ref="P46:Q46"/>
+    <mergeCell ref="P47:Q47"/>
+    <mergeCell ref="P43:Q43"/>
     <mergeCell ref="J42:K44"/>
     <mergeCell ref="AF37:AF38"/>
     <mergeCell ref="AF6:AK6"/>
@@ -4097,14 +4080,31 @@
     <mergeCell ref="Z9:Z15"/>
     <mergeCell ref="T12:T18"/>
     <mergeCell ref="H6:M6"/>
-    <mergeCell ref="P48:Q48"/>
-    <mergeCell ref="P49:Q49"/>
-    <mergeCell ref="P42:Q42"/>
-    <mergeCell ref="P44:Q44"/>
-    <mergeCell ref="P45:Q45"/>
-    <mergeCell ref="P46:Q46"/>
-    <mergeCell ref="P47:Q47"/>
-    <mergeCell ref="P43:Q43"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="N9:N15"/>
+    <mergeCell ref="H12:H18"/>
+    <mergeCell ref="N16:N22"/>
+    <mergeCell ref="H19:H25"/>
+    <mergeCell ref="N23:N29"/>
+    <mergeCell ref="H26:H32"/>
+    <mergeCell ref="N30:N35"/>
+    <mergeCell ref="H33:H38"/>
+    <mergeCell ref="N36:S38"/>
+    <mergeCell ref="T8:T11"/>
+    <mergeCell ref="AL38:AQ38"/>
+    <mergeCell ref="AL6:AQ6"/>
+    <mergeCell ref="AL8:AL12"/>
+    <mergeCell ref="AL13:AL19"/>
+    <mergeCell ref="AN13:AO13"/>
+    <mergeCell ref="AL20:AL26"/>
+    <mergeCell ref="AL27:AL33"/>
+    <mergeCell ref="AL34:AL37"/>
+    <mergeCell ref="T19:T25"/>
+    <mergeCell ref="Z23:Z29"/>
+    <mergeCell ref="T26:T32"/>
+    <mergeCell ref="Z30:Z35"/>
+    <mergeCell ref="Z16:Z22"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4124,15 +4124,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100862694ECED4E1948B5E8D6F6BADC8D0D" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="ae739b22c1d0ad2d0a68cf71a23d442c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="102bceca-7b01-449b-a089-7caeaaf28d79" xmlns:ns3="7fc2edd5-909c-43a2-b3b4-2537dcd3eee1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="05a22d24dcf35b0ff3f755cd1ef480a8" ns2:_="" ns3:_="">
     <xsd:import namespace="102bceca-7b01-449b-a089-7caeaaf28d79"/>
@@ -4333,6 +4324,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{027A5389-2971-44C0-A0D1-6195B9A552F9}">
   <ds:schemaRefs>
@@ -4351,14 +4351,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23969816-9B9E-4320-B349-9EB0D8911C7F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4F02508-5572-4BFA-B015-F122D6CC4035}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4375,4 +4367,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23969816-9B9E-4320-B349-9EB0D8911C7F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>